<commit_message>
empezamos tema 3 en caucasia
</commit_message>
<xml_diff>
--- a/9_asistencia_evaluacion/pivu_caucasia.xlsx
+++ b/9_asistencia_evaluacion/pivu_caucasia.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\marco\Documentos\extension\camino-udea\9_asistencia_evaluacion\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA2ADC41-D391-4381-B7DF-3B2B8F439A0E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B705A49-5EC7-4F44-8B6D-88E1C56CDFB6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -3052,14 +3052,14 @@
         <v>1041633525</v>
       </c>
       <c r="D8" s="13">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E8" s="13"/>
       <c r="F8" s="13"/>
       <c r="G8" s="13"/>
       <c r="H8" s="32">
         <f t="shared" si="0"/>
-        <v>0.25</v>
+        <v>0.5</v>
       </c>
       <c r="I8" s="33"/>
       <c r="J8" s="33"/>
@@ -3376,14 +3376,14 @@
         <v>1038111245</v>
       </c>
       <c r="D14" s="13">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E14" s="13"/>
       <c r="F14" s="13"/>
       <c r="G14" s="13"/>
       <c r="H14" s="32">
         <f t="shared" si="0"/>
-        <v>1</v>
+        <v>1.25</v>
       </c>
       <c r="I14" s="33"/>
       <c r="J14" s="33"/>
@@ -3431,14 +3431,14 @@
         <v>1038134078</v>
       </c>
       <c r="D15" s="13">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E15" s="13"/>
       <c r="F15" s="13"/>
       <c r="G15" s="13"/>
       <c r="H15" s="32">
         <f t="shared" si="0"/>
-        <v>0.25</v>
+        <v>0</v>
       </c>
       <c r="I15" s="33"/>
       <c r="J15" s="33"/>
@@ -3485,7 +3485,9 @@
         <f>+Inscritos!D14</f>
         <v>1038647898</v>
       </c>
-      <c r="D16" s="13"/>
+      <c r="D16" s="13">
+        <v>0</v>
+      </c>
       <c r="E16" s="13"/>
       <c r="F16" s="13"/>
       <c r="G16" s="13"/>
@@ -3591,7 +3593,9 @@
         <f>+Inscritos!D16</f>
         <v>1038109330</v>
       </c>
-      <c r="D18" s="13"/>
+      <c r="D18" s="13">
+        <v>0</v>
+      </c>
       <c r="E18" s="13"/>
       <c r="F18" s="13"/>
       <c r="G18" s="13"/>
@@ -3644,7 +3648,9 @@
         <f>+Inscritos!D17</f>
         <v>1038647796</v>
       </c>
-      <c r="D19" s="13"/>
+      <c r="D19" s="13">
+        <v>0</v>
+      </c>
       <c r="E19" s="13"/>
       <c r="F19" s="13"/>
       <c r="G19" s="13"/>
@@ -3698,14 +3704,14 @@
         <v>1038105559</v>
       </c>
       <c r="D20" s="13">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E20" s="13"/>
       <c r="F20" s="13"/>
       <c r="G20" s="13"/>
       <c r="H20" s="32">
         <f t="shared" si="0"/>
-        <v>0.25</v>
+        <v>0.5</v>
       </c>
       <c r="I20" s="33"/>
       <c r="J20" s="33"/>
@@ -4127,13 +4133,15 @@
         <f>+Inscritos!D26</f>
         <v>1038115554</v>
       </c>
-      <c r="D28" s="13"/>
+      <c r="D28" s="13">
+        <v>1</v>
+      </c>
       <c r="E28" s="13"/>
       <c r="F28" s="13"/>
       <c r="G28" s="13"/>
       <c r="H28" s="32">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>0.25</v>
       </c>
       <c r="I28" s="33"/>
       <c r="J28" s="33"/>
@@ -4344,14 +4352,14 @@
         <v>1038104210</v>
       </c>
       <c r="D32" s="13">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E32" s="13"/>
       <c r="F32" s="13"/>
       <c r="G32" s="13"/>
       <c r="H32" s="32">
         <f t="shared" si="0"/>
-        <v>1.25</v>
+        <v>1.5</v>
       </c>
       <c r="I32" s="33"/>
       <c r="J32" s="33"/>
@@ -4507,14 +4515,14 @@
         <v>1038115337</v>
       </c>
       <c r="D35" s="13">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E35" s="13"/>
       <c r="F35" s="13"/>
       <c r="G35" s="13"/>
       <c r="H35" s="32">
         <f t="shared" si="0"/>
-        <v>0.25</v>
+        <v>0.5</v>
       </c>
       <c r="I35" s="33"/>
       <c r="J35" s="33"/>

</xml_diff>

<commit_message>
estrategia de secuencias listo
</commit_message>
<xml_diff>
--- a/9_asistencia_evaluacion/pivu_caucasia.xlsx
+++ b/9_asistencia_evaluacion/pivu_caucasia.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\marco\Documentos\extension\camino-udea\9_asistencia_evaluacion\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B705A49-5EC7-4F44-8B6D-88E1C56CDFB6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A57E7318-1D14-44DF-B70A-12894F39A093}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -871,7 +871,7 @@
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="43" fontId="11" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="144">
+  <cellXfs count="145">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1133,6 +1133,90 @@
     <xf numFmtId="0" fontId="22" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="14" fillId="11" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1160,15 +1244,6 @@
     <xf numFmtId="0" fontId="3" fillId="7" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="9" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1211,79 +1286,7 @@
     <xf numFmtId="0" fontId="3" fillId="6" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="8" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="9" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="8" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="9" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="9" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="9" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="9" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="9" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="9" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -2998,12 +3001,14 @@
         <f>+Inscritos!D5</f>
         <v>1038117202</v>
       </c>
-      <c r="D7" s="13"/>
+      <c r="D7" s="13">
+        <v>0</v>
+      </c>
       <c r="E7" s="13"/>
       <c r="F7" s="13"/>
       <c r="G7" s="13"/>
       <c r="H7" s="32">
-        <f t="shared" ref="H7:H39" si="0">+SUM(D7:G7)/4</f>
+        <f t="shared" ref="H7:H40" si="0">+SUM(D7:G7)/4</f>
         <v>0</v>
       </c>
       <c r="I7" s="33"/>
@@ -3052,14 +3057,14 @@
         <v>1041633525</v>
       </c>
       <c r="D8" s="13">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E8" s="13"/>
       <c r="F8" s="13"/>
       <c r="G8" s="13"/>
       <c r="H8" s="32">
         <f t="shared" si="0"/>
-        <v>0.5</v>
+        <v>0.75</v>
       </c>
       <c r="I8" s="33"/>
       <c r="J8" s="33"/>
@@ -3106,7 +3111,9 @@
         <f>+Inscritos!D7</f>
         <v>1038648794</v>
       </c>
-      <c r="D9" s="13"/>
+      <c r="D9" s="13">
+        <v>0</v>
+      </c>
       <c r="E9" s="13"/>
       <c r="F9" s="13"/>
       <c r="G9" s="13"/>
@@ -3215,14 +3222,14 @@
         <v>1038110143</v>
       </c>
       <c r="D11" s="13">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E11" s="13"/>
       <c r="F11" s="13"/>
       <c r="G11" s="13"/>
       <c r="H11" s="32">
         <f t="shared" si="0"/>
-        <v>0.25</v>
+        <v>0.5</v>
       </c>
       <c r="I11" s="33"/>
       <c r="J11" s="33"/>
@@ -3269,7 +3276,9 @@
         <f>+Inscritos!D10</f>
         <v>1038114008</v>
       </c>
-      <c r="D12" s="13"/>
+      <c r="D12" s="13">
+        <v>0</v>
+      </c>
       <c r="E12" s="13"/>
       <c r="F12" s="13"/>
       <c r="G12" s="13"/>
@@ -3322,7 +3331,9 @@
         <f>+Inscritos!D11</f>
         <v>1038116790</v>
       </c>
-      <c r="D13" s="13"/>
+      <c r="D13" s="13">
+        <v>0</v>
+      </c>
       <c r="E13" s="13"/>
       <c r="F13" s="13"/>
       <c r="G13" s="13"/>
@@ -3376,14 +3387,14 @@
         <v>1038111245</v>
       </c>
       <c r="D14" s="13">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E14" s="13"/>
       <c r="F14" s="13"/>
       <c r="G14" s="13"/>
       <c r="H14" s="32">
         <f t="shared" si="0"/>
-        <v>1.25</v>
+        <v>1.5</v>
       </c>
       <c r="I14" s="33"/>
       <c r="J14" s="33"/>
@@ -3431,14 +3442,14 @@
         <v>1038134078</v>
       </c>
       <c r="D15" s="13">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E15" s="13"/>
       <c r="F15" s="13"/>
       <c r="G15" s="13"/>
       <c r="H15" s="32">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>0.25</v>
       </c>
       <c r="I15" s="33"/>
       <c r="J15" s="33"/>
@@ -3540,13 +3551,15 @@
         <f>+Inscritos!D15</f>
         <v>1038112414</v>
       </c>
-      <c r="D17" s="13"/>
+      <c r="D17" s="13">
+        <v>1</v>
+      </c>
       <c r="E17" s="13"/>
       <c r="F17" s="13"/>
       <c r="G17" s="13"/>
       <c r="H17" s="32">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>0.25</v>
       </c>
       <c r="I17" s="33"/>
       <c r="J17" s="33"/>
@@ -3704,14 +3717,14 @@
         <v>1038105559</v>
       </c>
       <c r="D20" s="13">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E20" s="13"/>
       <c r="F20" s="13"/>
       <c r="G20" s="13"/>
       <c r="H20" s="32">
         <f t="shared" si="0"/>
-        <v>0.5</v>
+        <v>0.75</v>
       </c>
       <c r="I20" s="33"/>
       <c r="J20" s="33"/>
@@ -3758,13 +3771,15 @@
         <f>+Inscritos!D19</f>
         <v>1011513720</v>
       </c>
-      <c r="D21" s="13"/>
+      <c r="D21" s="13">
+        <v>1</v>
+      </c>
       <c r="E21" s="13"/>
       <c r="F21" s="13"/>
       <c r="G21" s="13"/>
       <c r="H21" s="32">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>0.25</v>
       </c>
       <c r="I21" s="33"/>
       <c r="J21" s="33"/>
@@ -3811,13 +3826,15 @@
         <f>+Inscritos!D20</f>
         <v>1038114154</v>
       </c>
-      <c r="D22" s="13"/>
+      <c r="D22" s="13">
+        <v>1</v>
+      </c>
       <c r="E22" s="13"/>
       <c r="F22" s="13"/>
       <c r="G22" s="13"/>
       <c r="H22" s="32">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>0.25</v>
       </c>
       <c r="I22" s="33"/>
       <c r="J22" s="33"/>
@@ -3972,13 +3989,15 @@
         <f>+Inscritos!D23</f>
         <v>1073690694</v>
       </c>
-      <c r="D25" s="13"/>
+      <c r="D25" s="13">
+        <v>1</v>
+      </c>
       <c r="E25" s="13"/>
       <c r="F25" s="13"/>
       <c r="G25" s="13"/>
       <c r="H25" s="32">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>0.25</v>
       </c>
       <c r="I25" s="33"/>
       <c r="J25" s="33"/>
@@ -4079,14 +4098,14 @@
         <v>1038114203</v>
       </c>
       <c r="D27" s="13">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E27" s="13"/>
       <c r="F27" s="13"/>
       <c r="G27" s="13"/>
       <c r="H27" s="32">
         <f t="shared" si="0"/>
-        <v>0.25</v>
+        <v>0.5</v>
       </c>
       <c r="I27" s="33"/>
       <c r="J27" s="33"/>
@@ -4189,14 +4208,14 @@
         <v>1038109706</v>
       </c>
       <c r="D29" s="13">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E29" s="13"/>
       <c r="F29" s="13"/>
       <c r="G29" s="13"/>
       <c r="H29" s="32">
         <f t="shared" si="0"/>
-        <v>0.75</v>
+        <v>1</v>
       </c>
       <c r="I29" s="33"/>
       <c r="J29" s="33"/>
@@ -4298,13 +4317,15 @@
         <f>+Inscritos!D29</f>
         <v>1038112417</v>
       </c>
-      <c r="D31" s="56"/>
+      <c r="D31" s="56">
+        <v>1</v>
+      </c>
       <c r="E31" s="13"/>
       <c r="F31" s="13"/>
       <c r="G31" s="13"/>
       <c r="H31" s="32">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>0.25</v>
       </c>
       <c r="I31" s="33"/>
       <c r="J31" s="33"/>
@@ -4352,14 +4373,14 @@
         <v>1038104210</v>
       </c>
       <c r="D32" s="13">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E32" s="13"/>
       <c r="F32" s="13"/>
       <c r="G32" s="13"/>
       <c r="H32" s="32">
         <f t="shared" si="0"/>
-        <v>1.5</v>
+        <v>1.75</v>
       </c>
       <c r="I32" s="33"/>
       <c r="J32" s="33"/>
@@ -4407,14 +4428,14 @@
         <v>1100016222</v>
       </c>
       <c r="D33" s="13">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E33" s="13"/>
       <c r="F33" s="13"/>
       <c r="G33" s="13"/>
       <c r="H33" s="32">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>0.25</v>
       </c>
       <c r="I33" s="33"/>
       <c r="J33" s="33"/>
@@ -4461,13 +4482,15 @@
         <f>+Inscritos!D32</f>
         <v>1038111917</v>
       </c>
-      <c r="D34" s="13"/>
+      <c r="D34" s="13">
+        <v>1</v>
+      </c>
       <c r="E34" s="13"/>
       <c r="F34" s="13"/>
       <c r="G34" s="13"/>
       <c r="H34" s="32">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>0.25</v>
       </c>
       <c r="I34" s="33"/>
       <c r="J34" s="33"/>
@@ -4515,14 +4538,14 @@
         <v>1038115337</v>
       </c>
       <c r="D35" s="13">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E35" s="13"/>
       <c r="F35" s="13"/>
       <c r="G35" s="13"/>
       <c r="H35" s="32">
         <f t="shared" si="0"/>
-        <v>0.5</v>
+        <v>0.75</v>
       </c>
       <c r="I35" s="33"/>
       <c r="J35" s="33"/>
@@ -4624,13 +4647,15 @@
         <f>+Inscritos!D35</f>
         <v>1125368371</v>
       </c>
-      <c r="D37" s="13"/>
+      <c r="D37" s="13">
+        <v>1</v>
+      </c>
       <c r="E37" s="13"/>
       <c r="F37" s="13"/>
       <c r="G37" s="13"/>
       <c r="H37" s="32">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>0.25</v>
       </c>
       <c r="I37" s="33"/>
       <c r="J37" s="33"/>
@@ -4678,14 +4703,14 @@
         <v>1038104997</v>
       </c>
       <c r="D38" s="13">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E38" s="13"/>
       <c r="F38" s="13"/>
       <c r="G38" s="13"/>
       <c r="H38" s="32">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>0.25</v>
       </c>
       <c r="I38" s="33"/>
       <c r="J38" s="33"/>
@@ -4732,13 +4757,15 @@
         <f>+Inscritos!D37</f>
         <v>1038113397</v>
       </c>
-      <c r="D39" s="13"/>
+      <c r="D39" s="13">
+        <v>1</v>
+      </c>
       <c r="E39" s="13"/>
       <c r="F39" s="13"/>
       <c r="G39" s="13"/>
       <c r="H39" s="32">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>0.25</v>
       </c>
       <c r="I39" s="33"/>
       <c r="J39" s="33"/>
@@ -4779,6 +4806,13 @@
       </c>
       <c r="B40" t="s">
         <v>105</v>
+      </c>
+      <c r="D40" s="144">
+        <v>0</v>
+      </c>
+      <c r="H40" s="2">
+        <f t="shared" si="0"/>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -4833,30 +4867,30 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:20" ht="72.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B1" s="119" t="s">
+      <c r="B1" s="93" t="s">
         <v>18</v>
       </c>
-      <c r="C1" s="119"/>
-      <c r="D1" s="119"/>
-      <c r="E1" s="119"/>
-      <c r="F1" s="119"/>
-      <c r="G1" s="119"/>
-      <c r="H1" s="119"/>
-      <c r="I1" s="119"/>
-      <c r="J1" s="119"/>
-      <c r="K1" s="119"/>
-      <c r="L1" s="119"/>
-      <c r="M1" s="119"/>
-      <c r="N1" s="119"/>
-      <c r="O1" s="119"/>
-      <c r="P1" s="119"/>
-      <c r="Q1" s="119"/>
-      <c r="R1" s="119"/>
-      <c r="S1" s="119"/>
-      <c r="T1" s="119"/>
+      <c r="C1" s="93"/>
+      <c r="D1" s="93"/>
+      <c r="E1" s="93"/>
+      <c r="F1" s="93"/>
+      <c r="G1" s="93"/>
+      <c r="H1" s="93"/>
+      <c r="I1" s="93"/>
+      <c r="J1" s="93"/>
+      <c r="K1" s="93"/>
+      <c r="L1" s="93"/>
+      <c r="M1" s="93"/>
+      <c r="N1" s="93"/>
+      <c r="O1" s="93"/>
+      <c r="P1" s="93"/>
+      <c r="Q1" s="93"/>
+      <c r="R1" s="93"/>
+      <c r="S1" s="93"/>
+      <c r="T1" s="93"/>
     </row>
     <row r="2" spans="1:20" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A2" s="105" t="s">
+      <c r="A2" s="130" t="s">
         <v>13</v>
       </c>
       <c r="B2" s="89" t="s">
@@ -4865,89 +4899,89 @@
       <c r="C2" s="65" t="s">
         <v>3</v>
       </c>
-      <c r="D2" s="93" t="str">
+      <c r="D2" s="121" t="str">
         <f>Asistencia!D2</f>
         <v>NOMBRE DOCENTE</v>
       </c>
-      <c r="E2" s="94"/>
-      <c r="F2" s="95"/>
-      <c r="G2" s="93" t="str">
+      <c r="E2" s="122"/>
+      <c r="F2" s="123"/>
+      <c r="G2" s="121" t="str">
         <f>Asistencia!I2</f>
         <v>NOMBRE DOCENTE</v>
       </c>
-      <c r="H2" s="94"/>
-      <c r="I2" s="94"/>
-      <c r="J2" s="94"/>
-      <c r="K2" s="95"/>
-      <c r="L2" s="93" t="s">
+      <c r="H2" s="122"/>
+      <c r="I2" s="122"/>
+      <c r="J2" s="122"/>
+      <c r="K2" s="123"/>
+      <c r="L2" s="121" t="s">
         <v>19</v>
       </c>
-      <c r="M2" s="94"/>
-      <c r="N2" s="94"/>
-      <c r="O2" s="94"/>
-      <c r="P2" s="95"/>
-      <c r="Q2" s="93" t="str">
+      <c r="M2" s="122"/>
+      <c r="N2" s="122"/>
+      <c r="O2" s="122"/>
+      <c r="P2" s="123"/>
+      <c r="Q2" s="121" t="str">
         <f>Asistencia!AA2</f>
         <v>NOMBRE DOCENTE</v>
       </c>
-      <c r="R2" s="94"/>
-      <c r="S2" s="94"/>
-      <c r="T2" s="95"/>
+      <c r="R2" s="122"/>
+      <c r="S2" s="122"/>
+      <c r="T2" s="123"/>
     </row>
     <row r="3" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="106"/>
+      <c r="A3" s="131"/>
       <c r="B3" s="90"/>
       <c r="C3" s="66"/>
-      <c r="D3" s="113" t="s">
+      <c r="D3" s="138" t="s">
         <v>7</v>
       </c>
-      <c r="E3" s="114"/>
-      <c r="F3" s="115"/>
-      <c r="G3" s="107" t="s">
+      <c r="E3" s="139"/>
+      <c r="F3" s="140"/>
+      <c r="G3" s="132" t="s">
         <v>2</v>
       </c>
-      <c r="H3" s="108"/>
-      <c r="I3" s="108"/>
-      <c r="J3" s="108"/>
-      <c r="K3" s="109"/>
-      <c r="L3" s="138" t="s">
+      <c r="H3" s="133"/>
+      <c r="I3" s="133"/>
+      <c r="J3" s="133"/>
+      <c r="K3" s="134"/>
+      <c r="L3" s="115" t="s">
         <v>1</v>
       </c>
-      <c r="M3" s="139"/>
-      <c r="N3" s="139"/>
-      <c r="O3" s="139"/>
-      <c r="P3" s="140"/>
-      <c r="Q3" s="96" t="s">
-        <v>0</v>
-      </c>
-      <c r="R3" s="97"/>
-      <c r="S3" s="97"/>
-      <c r="T3" s="98"/>
+      <c r="M3" s="116"/>
+      <c r="N3" s="116"/>
+      <c r="O3" s="116"/>
+      <c r="P3" s="117"/>
+      <c r="Q3" s="124" t="s">
+        <v>0</v>
+      </c>
+      <c r="R3" s="125"/>
+      <c r="S3" s="125"/>
+      <c r="T3" s="126"/>
     </row>
     <row r="4" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="106"/>
+      <c r="A4" s="131"/>
       <c r="B4" s="90"/>
       <c r="C4" s="66"/>
-      <c r="D4" s="116"/>
-      <c r="E4" s="117"/>
-      <c r="F4" s="118"/>
-      <c r="G4" s="110"/>
-      <c r="H4" s="111"/>
-      <c r="I4" s="111"/>
-      <c r="J4" s="111"/>
-      <c r="K4" s="112"/>
-      <c r="L4" s="141"/>
-      <c r="M4" s="142"/>
-      <c r="N4" s="142"/>
-      <c r="O4" s="142"/>
-      <c r="P4" s="143"/>
-      <c r="Q4" s="99"/>
-      <c r="R4" s="100"/>
-      <c r="S4" s="100"/>
-      <c r="T4" s="101"/>
+      <c r="D4" s="141"/>
+      <c r="E4" s="142"/>
+      <c r="F4" s="143"/>
+      <c r="G4" s="135"/>
+      <c r="H4" s="136"/>
+      <c r="I4" s="136"/>
+      <c r="J4" s="136"/>
+      <c r="K4" s="137"/>
+      <c r="L4" s="118"/>
+      <c r="M4" s="119"/>
+      <c r="N4" s="119"/>
+      <c r="O4" s="119"/>
+      <c r="P4" s="120"/>
+      <c r="Q4" s="127"/>
+      <c r="R4" s="128"/>
+      <c r="S4" s="128"/>
+      <c r="T4" s="129"/>
     </row>
     <row r="5" spans="1:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="106"/>
+      <c r="A5" s="131"/>
       <c r="B5" s="90"/>
       <c r="C5" s="66"/>
       <c r="D5" s="17">
@@ -7523,186 +7557,195 @@
       </c>
     </row>
     <row r="66" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="D66" s="123" t="s">
+      <c r="D66" s="97" t="s">
         <v>24</v>
       </c>
-      <c r="E66" s="126" t="s">
+      <c r="E66" s="100" t="s">
         <v>12</v>
       </c>
-      <c r="G66" s="120" t="s">
+      <c r="G66" s="94" t="s">
         <v>8</v>
       </c>
-      <c r="H66" s="132" t="s">
+      <c r="H66" s="109" t="s">
         <v>9</v>
       </c>
-      <c r="I66" s="132" t="s">
+      <c r="I66" s="109" t="s">
         <v>10</v>
       </c>
-      <c r="J66" s="120" t="s">
+      <c r="J66" s="94" t="s">
         <v>11</v>
       </c>
-      <c r="L66" s="102" t="s">
+      <c r="L66" s="103" t="s">
         <v>8</v>
       </c>
-      <c r="M66" s="129" t="s">
+      <c r="M66" s="106" t="s">
         <v>9</v>
       </c>
-      <c r="N66" s="129" t="s">
+      <c r="N66" s="106" t="s">
         <v>10</v>
       </c>
-      <c r="O66" s="102" t="s">
+      <c r="O66" s="103" t="s">
         <v>11</v>
       </c>
-      <c r="Q66" s="135" t="s">
+      <c r="Q66" s="112" t="s">
         <v>24</v>
       </c>
-      <c r="R66" s="135" t="s">
+      <c r="R66" s="112" t="s">
         <v>4</v>
       </c>
-      <c r="S66" s="135" t="s">
+      <c r="S66" s="112" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="67" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="D67" s="124"/>
-      <c r="E67" s="127"/>
-      <c r="G67" s="121"/>
-      <c r="H67" s="133"/>
-      <c r="I67" s="133"/>
-      <c r="J67" s="121"/>
-      <c r="L67" s="103"/>
-      <c r="M67" s="130"/>
-      <c r="N67" s="130"/>
-      <c r="O67" s="103"/>
-      <c r="Q67" s="136"/>
-      <c r="R67" s="136"/>
-      <c r="S67" s="136"/>
+      <c r="D67" s="98"/>
+      <c r="E67" s="101"/>
+      <c r="G67" s="95"/>
+      <c r="H67" s="110"/>
+      <c r="I67" s="110"/>
+      <c r="J67" s="95"/>
+      <c r="L67" s="104"/>
+      <c r="M67" s="107"/>
+      <c r="N67" s="107"/>
+      <c r="O67" s="104"/>
+      <c r="Q67" s="113"/>
+      <c r="R67" s="113"/>
+      <c r="S67" s="113"/>
     </row>
     <row r="68" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="D68" s="124"/>
-      <c r="E68" s="127"/>
-      <c r="G68" s="121"/>
-      <c r="H68" s="133"/>
-      <c r="I68" s="133"/>
-      <c r="J68" s="121"/>
-      <c r="L68" s="103"/>
-      <c r="M68" s="130"/>
-      <c r="N68" s="130"/>
-      <c r="O68" s="103"/>
-      <c r="Q68" s="136"/>
-      <c r="R68" s="136"/>
-      <c r="S68" s="136"/>
+      <c r="D68" s="98"/>
+      <c r="E68" s="101"/>
+      <c r="G68" s="95"/>
+      <c r="H68" s="110"/>
+      <c r="I68" s="110"/>
+      <c r="J68" s="95"/>
+      <c r="L68" s="104"/>
+      <c r="M68" s="107"/>
+      <c r="N68" s="107"/>
+      <c r="O68" s="104"/>
+      <c r="Q68" s="113"/>
+      <c r="R68" s="113"/>
+      <c r="S68" s="113"/>
     </row>
     <row r="69" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="D69" s="124"/>
-      <c r="E69" s="127"/>
-      <c r="G69" s="121"/>
-      <c r="H69" s="133"/>
-      <c r="I69" s="133"/>
-      <c r="J69" s="121"/>
-      <c r="L69" s="103"/>
-      <c r="M69" s="130"/>
-      <c r="N69" s="130"/>
-      <c r="O69" s="103"/>
-      <c r="Q69" s="136"/>
-      <c r="R69" s="136"/>
-      <c r="S69" s="136"/>
+      <c r="D69" s="98"/>
+      <c r="E69" s="101"/>
+      <c r="G69" s="95"/>
+      <c r="H69" s="110"/>
+      <c r="I69" s="110"/>
+      <c r="J69" s="95"/>
+      <c r="L69" s="104"/>
+      <c r="M69" s="107"/>
+      <c r="N69" s="107"/>
+      <c r="O69" s="104"/>
+      <c r="Q69" s="113"/>
+      <c r="R69" s="113"/>
+      <c r="S69" s="113"/>
     </row>
     <row r="70" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="D70" s="124"/>
-      <c r="E70" s="127"/>
-      <c r="G70" s="121"/>
-      <c r="H70" s="133"/>
-      <c r="I70" s="133"/>
-      <c r="J70" s="121"/>
-      <c r="L70" s="103"/>
-      <c r="M70" s="130"/>
-      <c r="N70" s="130"/>
-      <c r="O70" s="103"/>
-      <c r="Q70" s="136"/>
-      <c r="R70" s="136"/>
-      <c r="S70" s="136"/>
+      <c r="D70" s="98"/>
+      <c r="E70" s="101"/>
+      <c r="G70" s="95"/>
+      <c r="H70" s="110"/>
+      <c r="I70" s="110"/>
+      <c r="J70" s="95"/>
+      <c r="L70" s="104"/>
+      <c r="M70" s="107"/>
+      <c r="N70" s="107"/>
+      <c r="O70" s="104"/>
+      <c r="Q70" s="113"/>
+      <c r="R70" s="113"/>
+      <c r="S70" s="113"/>
     </row>
     <row r="71" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="D71" s="124"/>
-      <c r="E71" s="127"/>
-      <c r="G71" s="121"/>
-      <c r="H71" s="133"/>
-      <c r="I71" s="133"/>
-      <c r="J71" s="121"/>
-      <c r="L71" s="103"/>
-      <c r="M71" s="130"/>
-      <c r="N71" s="130"/>
-      <c r="O71" s="103"/>
-      <c r="Q71" s="136"/>
-      <c r="R71" s="136"/>
-      <c r="S71" s="136"/>
+      <c r="D71" s="98"/>
+      <c r="E71" s="101"/>
+      <c r="G71" s="95"/>
+      <c r="H71" s="110"/>
+      <c r="I71" s="110"/>
+      <c r="J71" s="95"/>
+      <c r="L71" s="104"/>
+      <c r="M71" s="107"/>
+      <c r="N71" s="107"/>
+      <c r="O71" s="104"/>
+      <c r="Q71" s="113"/>
+      <c r="R71" s="113"/>
+      <c r="S71" s="113"/>
     </row>
     <row r="72" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="D72" s="124"/>
-      <c r="E72" s="127"/>
-      <c r="G72" s="121"/>
-      <c r="H72" s="133"/>
-      <c r="I72" s="133"/>
-      <c r="J72" s="121"/>
-      <c r="L72" s="103"/>
-      <c r="M72" s="130"/>
-      <c r="N72" s="130"/>
-      <c r="O72" s="103"/>
-      <c r="Q72" s="136"/>
-      <c r="R72" s="136"/>
-      <c r="S72" s="136"/>
+      <c r="D72" s="98"/>
+      <c r="E72" s="101"/>
+      <c r="G72" s="95"/>
+      <c r="H72" s="110"/>
+      <c r="I72" s="110"/>
+      <c r="J72" s="95"/>
+      <c r="L72" s="104"/>
+      <c r="M72" s="107"/>
+      <c r="N72" s="107"/>
+      <c r="O72" s="104"/>
+      <c r="Q72" s="113"/>
+      <c r="R72" s="113"/>
+      <c r="S72" s="113"/>
     </row>
     <row r="73" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="D73" s="124"/>
-      <c r="E73" s="127"/>
-      <c r="G73" s="121"/>
-      <c r="H73" s="133"/>
-      <c r="I73" s="133"/>
-      <c r="J73" s="121"/>
-      <c r="L73" s="103"/>
-      <c r="M73" s="130"/>
-      <c r="N73" s="130"/>
-      <c r="O73" s="103"/>
-      <c r="Q73" s="136"/>
-      <c r="R73" s="136"/>
-      <c r="S73" s="136"/>
+      <c r="D73" s="98"/>
+      <c r="E73" s="101"/>
+      <c r="G73" s="95"/>
+      <c r="H73" s="110"/>
+      <c r="I73" s="110"/>
+      <c r="J73" s="95"/>
+      <c r="L73" s="104"/>
+      <c r="M73" s="107"/>
+      <c r="N73" s="107"/>
+      <c r="O73" s="104"/>
+      <c r="Q73" s="113"/>
+      <c r="R73" s="113"/>
+      <c r="S73" s="113"/>
     </row>
     <row r="74" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="D74" s="124"/>
-      <c r="E74" s="127"/>
-      <c r="G74" s="121"/>
-      <c r="H74" s="133"/>
-      <c r="I74" s="133"/>
-      <c r="J74" s="121"/>
-      <c r="L74" s="103"/>
-      <c r="M74" s="130"/>
-      <c r="N74" s="130"/>
-      <c r="O74" s="103"/>
-      <c r="Q74" s="136"/>
-      <c r="R74" s="136"/>
-      <c r="S74" s="136"/>
+      <c r="D74" s="98"/>
+      <c r="E74" s="101"/>
+      <c r="G74" s="95"/>
+      <c r="H74" s="110"/>
+      <c r="I74" s="110"/>
+      <c r="J74" s="95"/>
+      <c r="L74" s="104"/>
+      <c r="M74" s="107"/>
+      <c r="N74" s="107"/>
+      <c r="O74" s="104"/>
+      <c r="Q74" s="113"/>
+      <c r="R74" s="113"/>
+      <c r="S74" s="113"/>
     </row>
     <row r="75" spans="1:20" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="D75" s="125"/>
-      <c r="E75" s="128"/>
-      <c r="G75" s="122"/>
-      <c r="H75" s="134"/>
-      <c r="I75" s="134"/>
-      <c r="J75" s="122"/>
-      <c r="L75" s="104"/>
-      <c r="M75" s="131"/>
-      <c r="N75" s="131"/>
-      <c r="O75" s="104"/>
-      <c r="Q75" s="137"/>
-      <c r="R75" s="137"/>
-      <c r="S75" s="137"/>
+      <c r="D75" s="99"/>
+      <c r="E75" s="102"/>
+      <c r="G75" s="96"/>
+      <c r="H75" s="111"/>
+      <c r="I75" s="111"/>
+      <c r="J75" s="96"/>
+      <c r="L75" s="105"/>
+      <c r="M75" s="108"/>
+      <c r="N75" s="108"/>
+      <c r="O75" s="105"/>
+      <c r="Q75" s="114"/>
+      <c r="R75" s="114"/>
+      <c r="S75" s="114"/>
     </row>
   </sheetData>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B6:T60">
     <sortCondition ref="B6"/>
   </sortState>
   <mergeCells count="25">
+    <mergeCell ref="G2:K2"/>
+    <mergeCell ref="D2:F2"/>
+    <mergeCell ref="Q3:T4"/>
+    <mergeCell ref="O66:O75"/>
+    <mergeCell ref="A2:A5"/>
+    <mergeCell ref="G3:K4"/>
+    <mergeCell ref="D3:F4"/>
+    <mergeCell ref="B2:B5"/>
+    <mergeCell ref="C2:C5"/>
     <mergeCell ref="B1:T1"/>
     <mergeCell ref="J66:J75"/>
     <mergeCell ref="D66:D75"/>
@@ -7719,15 +7762,6 @@
     <mergeCell ref="I66:I75"/>
     <mergeCell ref="Q2:T2"/>
     <mergeCell ref="L2:P2"/>
-    <mergeCell ref="G2:K2"/>
-    <mergeCell ref="D2:F2"/>
-    <mergeCell ref="Q3:T4"/>
-    <mergeCell ref="O66:O75"/>
-    <mergeCell ref="A2:A5"/>
-    <mergeCell ref="G3:K4"/>
-    <mergeCell ref="D3:F4"/>
-    <mergeCell ref="B2:B5"/>
-    <mergeCell ref="C2:C5"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
mejprada la clase del tema 3
</commit_message>
<xml_diff>
--- a/9_asistencia_evaluacion/pivu_caucasia.xlsx
+++ b/9_asistencia_evaluacion/pivu_caucasia.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\marco\Documentos\extension\camino-udea\9_asistencia_evaluacion\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A57E7318-1D14-44DF-B70A-12894F39A093}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AC8DFFB4-A832-4176-84F5-A0EA65CEAD52}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Inscritos" sheetId="2" r:id="rId1"/>
@@ -1025,6 +1025,9 @@
     <xf numFmtId="0" fontId="28" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="19" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1133,6 +1136,84 @@
     <xf numFmtId="0" fontId="22" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="14" fillId="11" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="11" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1163,15 +1244,6 @@
     <xf numFmtId="0" fontId="7" fillId="6" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="9" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
     </xf>
@@ -1215,78 +1287,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="9" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="11" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="11" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1786,28 +1786,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="72" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="92" t="s">
+      <c r="A1" s="93" t="s">
         <v>27</v>
       </c>
-      <c r="B1" s="91"/>
-      <c r="C1" s="91"/>
-      <c r="D1" s="91"/>
-      <c r="E1" s="91"/>
-      <c r="F1" s="91"/>
-      <c r="G1" s="91"/>
-      <c r="H1" s="91"/>
+      <c r="B1" s="92"/>
+      <c r="C1" s="92"/>
+      <c r="D1" s="92"/>
+      <c r="E1" s="92"/>
+      <c r="F1" s="92"/>
+      <c r="G1" s="92"/>
+      <c r="H1" s="92"/>
     </row>
     <row r="2" spans="1:9" ht="19.8" x14ac:dyDescent="0.3">
-      <c r="A2" s="91" t="s">
+      <c r="A2" s="92" t="s">
         <v>26</v>
       </c>
-      <c r="B2" s="91"/>
-      <c r="C2" s="91"/>
-      <c r="D2" s="91"/>
-      <c r="E2" s="91"/>
-      <c r="F2" s="91"/>
-      <c r="G2" s="91"/>
-      <c r="H2" s="91"/>
+      <c r="B2" s="92"/>
+      <c r="C2" s="92"/>
+      <c r="D2" s="92"/>
+      <c r="E2" s="92"/>
+      <c r="F2" s="92"/>
+      <c r="G2" s="92"/>
+      <c r="H2" s="92"/>
       <c r="I2" s="50" t="s">
         <v>99</v>
       </c>
@@ -2729,172 +2729,172 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:31" ht="66" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B1" s="64" t="s">
+      <c r="B1" s="65" t="s">
         <v>18</v>
       </c>
-      <c r="C1" s="64"/>
-      <c r="D1" s="64"/>
-      <c r="E1" s="64"/>
-      <c r="F1" s="64"/>
-      <c r="G1" s="64"/>
-      <c r="H1" s="64"/>
-      <c r="I1" s="64"/>
-      <c r="J1" s="64"/>
-      <c r="K1" s="64"/>
-      <c r="L1" s="64"/>
-      <c r="M1" s="64"/>
-      <c r="N1" s="64"/>
-      <c r="O1" s="64"/>
-      <c r="P1" s="64"/>
-      <c r="Q1" s="64"/>
-      <c r="R1" s="64"/>
-      <c r="S1" s="64"/>
-      <c r="T1" s="64"/>
-      <c r="U1" s="64"/>
-      <c r="V1" s="64"/>
-      <c r="W1" s="64"/>
-      <c r="X1" s="64"/>
-      <c r="Y1" s="64"/>
-      <c r="Z1" s="64"/>
-      <c r="AA1" s="64"/>
-      <c r="AB1" s="64"/>
-      <c r="AC1" s="64"/>
-      <c r="AD1" s="64"/>
-      <c r="AE1" s="64"/>
+      <c r="C1" s="65"/>
+      <c r="D1" s="65"/>
+      <c r="E1" s="65"/>
+      <c r="F1" s="65"/>
+      <c r="G1" s="65"/>
+      <c r="H1" s="65"/>
+      <c r="I1" s="65"/>
+      <c r="J1" s="65"/>
+      <c r="K1" s="65"/>
+      <c r="L1" s="65"/>
+      <c r="M1" s="65"/>
+      <c r="N1" s="65"/>
+      <c r="O1" s="65"/>
+      <c r="P1" s="65"/>
+      <c r="Q1" s="65"/>
+      <c r="R1" s="65"/>
+      <c r="S1" s="65"/>
+      <c r="T1" s="65"/>
+      <c r="U1" s="65"/>
+      <c r="V1" s="65"/>
+      <c r="W1" s="65"/>
+      <c r="X1" s="65"/>
+      <c r="Y1" s="65"/>
+      <c r="Z1" s="65"/>
+      <c r="AA1" s="65"/>
+      <c r="AB1" s="65"/>
+      <c r="AC1" s="65"/>
+      <c r="AD1" s="65"/>
+      <c r="AE1" s="65"/>
     </row>
     <row r="2" spans="1:31" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A2" s="65" t="s">
+      <c r="A2" s="66" t="s">
         <v>13</v>
       </c>
-      <c r="B2" s="89" t="s">
+      <c r="B2" s="90" t="s">
         <v>21</v>
       </c>
-      <c r="C2" s="65" t="s">
+      <c r="C2" s="66" t="s">
         <v>3</v>
       </c>
-      <c r="D2" s="82" t="s">
+      <c r="D2" s="83" t="s">
         <v>19</v>
       </c>
-      <c r="E2" s="83"/>
-      <c r="F2" s="83"/>
-      <c r="G2" s="83"/>
-      <c r="H2" s="84"/>
-      <c r="I2" s="67" t="s">
+      <c r="E2" s="84"/>
+      <c r="F2" s="84"/>
+      <c r="G2" s="84"/>
+      <c r="H2" s="85"/>
+      <c r="I2" s="68" t="s">
         <v>19</v>
       </c>
-      <c r="J2" s="68"/>
-      <c r="K2" s="68"/>
-      <c r="L2" s="68"/>
-      <c r="M2" s="68"/>
-      <c r="N2" s="68"/>
-      <c r="O2" s="68"/>
-      <c r="P2" s="68"/>
-      <c r="Q2" s="69"/>
-      <c r="R2" s="76" t="s">
+      <c r="J2" s="69"/>
+      <c r="K2" s="69"/>
+      <c r="L2" s="69"/>
+      <c r="M2" s="69"/>
+      <c r="N2" s="69"/>
+      <c r="O2" s="69"/>
+      <c r="P2" s="69"/>
+      <c r="Q2" s="70"/>
+      <c r="R2" s="77" t="s">
         <v>19</v>
       </c>
-      <c r="S2" s="77"/>
-      <c r="T2" s="77"/>
-      <c r="U2" s="77"/>
-      <c r="V2" s="77"/>
-      <c r="W2" s="77"/>
-      <c r="X2" s="77"/>
-      <c r="Y2" s="77"/>
-      <c r="Z2" s="78"/>
-      <c r="AA2" s="57" t="s">
+      <c r="S2" s="78"/>
+      <c r="T2" s="78"/>
+      <c r="U2" s="78"/>
+      <c r="V2" s="78"/>
+      <c r="W2" s="78"/>
+      <c r="X2" s="78"/>
+      <c r="Y2" s="78"/>
+      <c r="Z2" s="79"/>
+      <c r="AA2" s="58" t="s">
         <v>19</v>
       </c>
-      <c r="AB2" s="58"/>
-      <c r="AC2" s="58"/>
-      <c r="AD2" s="58"/>
-      <c r="AE2" s="59"/>
+      <c r="AB2" s="59"/>
+      <c r="AC2" s="59"/>
+      <c r="AD2" s="59"/>
+      <c r="AE2" s="60"/>
     </row>
     <row r="3" spans="1:31" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="66"/>
-      <c r="B3" s="90"/>
-      <c r="C3" s="66"/>
-      <c r="D3" s="85" t="s">
+      <c r="A3" s="67"/>
+      <c r="B3" s="91"/>
+      <c r="C3" s="67"/>
+      <c r="D3" s="86" t="s">
         <v>7</v>
       </c>
-      <c r="E3" s="86"/>
-      <c r="F3" s="86"/>
-      <c r="G3" s="86"/>
-      <c r="H3" s="87"/>
-      <c r="I3" s="70" t="s">
+      <c r="E3" s="87"/>
+      <c r="F3" s="87"/>
+      <c r="G3" s="87"/>
+      <c r="H3" s="88"/>
+      <c r="I3" s="71" t="s">
         <v>2</v>
       </c>
-      <c r="J3" s="71"/>
-      <c r="K3" s="71"/>
-      <c r="L3" s="71"/>
-      <c r="M3" s="71"/>
-      <c r="N3" s="71"/>
-      <c r="O3" s="71"/>
-      <c r="P3" s="71"/>
-      <c r="Q3" s="72"/>
-      <c r="R3" s="79" t="s">
+      <c r="J3" s="72"/>
+      <c r="K3" s="72"/>
+      <c r="L3" s="72"/>
+      <c r="M3" s="72"/>
+      <c r="N3" s="72"/>
+      <c r="O3" s="72"/>
+      <c r="P3" s="72"/>
+      <c r="Q3" s="73"/>
+      <c r="R3" s="80" t="s">
         <v>1</v>
       </c>
-      <c r="S3" s="80"/>
-      <c r="T3" s="80"/>
-      <c r="U3" s="80"/>
-      <c r="V3" s="80"/>
-      <c r="W3" s="80"/>
-      <c r="X3" s="80"/>
-      <c r="Y3" s="80"/>
-      <c r="Z3" s="81"/>
-      <c r="AA3" s="60" t="s">
-        <v>0</v>
-      </c>
-      <c r="AB3" s="61"/>
-      <c r="AC3" s="61"/>
-      <c r="AD3" s="61"/>
-      <c r="AE3" s="62"/>
+      <c r="S3" s="81"/>
+      <c r="T3" s="81"/>
+      <c r="U3" s="81"/>
+      <c r="V3" s="81"/>
+      <c r="W3" s="81"/>
+      <c r="X3" s="81"/>
+      <c r="Y3" s="81"/>
+      <c r="Z3" s="82"/>
+      <c r="AA3" s="61" t="s">
+        <v>0</v>
+      </c>
+      <c r="AB3" s="62"/>
+      <c r="AC3" s="62"/>
+      <c r="AD3" s="62"/>
+      <c r="AE3" s="63"/>
     </row>
     <row r="4" spans="1:31" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="66"/>
-      <c r="B4" s="90"/>
-      <c r="C4" s="66"/>
-      <c r="D4" s="88" t="s">
+      <c r="A4" s="67"/>
+      <c r="B4" s="91"/>
+      <c r="C4" s="67"/>
+      <c r="D4" s="89" t="s">
         <v>22</v>
       </c>
-      <c r="E4" s="74"/>
-      <c r="F4" s="74"/>
-      <c r="G4" s="75"/>
+      <c r="E4" s="75"/>
+      <c r="F4" s="75"/>
+      <c r="G4" s="76"/>
       <c r="H4" s="1"/>
-      <c r="I4" s="73" t="s">
+      <c r="I4" s="74" t="s">
         <v>23</v>
       </c>
-      <c r="J4" s="74"/>
-      <c r="K4" s="74"/>
-      <c r="L4" s="74"/>
-      <c r="M4" s="74"/>
-      <c r="N4" s="74"/>
-      <c r="O4" s="74"/>
-      <c r="P4" s="75"/>
+      <c r="J4" s="75"/>
+      <c r="K4" s="75"/>
+      <c r="L4" s="75"/>
+      <c r="M4" s="75"/>
+      <c r="N4" s="75"/>
+      <c r="O4" s="75"/>
+      <c r="P4" s="76"/>
       <c r="Q4" s="3"/>
-      <c r="R4" s="73" t="s">
+      <c r="R4" s="74" t="s">
         <v>23</v>
       </c>
-      <c r="S4" s="74"/>
-      <c r="T4" s="74"/>
-      <c r="U4" s="74"/>
-      <c r="V4" s="74"/>
-      <c r="W4" s="74"/>
-      <c r="X4" s="74"/>
-      <c r="Y4" s="75"/>
+      <c r="S4" s="75"/>
+      <c r="T4" s="75"/>
+      <c r="U4" s="75"/>
+      <c r="V4" s="75"/>
+      <c r="W4" s="75"/>
+      <c r="X4" s="75"/>
+      <c r="Y4" s="76"/>
       <c r="Z4" s="12"/>
-      <c r="AA4" s="63" t="s">
+      <c r="AA4" s="64" t="s">
         <v>23</v>
       </c>
-      <c r="AB4" s="63"/>
-      <c r="AC4" s="63"/>
-      <c r="AD4" s="63"/>
+      <c r="AB4" s="64"/>
+      <c r="AC4" s="64"/>
+      <c r="AD4" s="64"/>
       <c r="AE4" s="3"/>
     </row>
     <row r="5" spans="1:31" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="66"/>
-      <c r="B5" s="90"/>
-      <c r="C5" s="66"/>
+      <c r="A5" s="67"/>
+      <c r="B5" s="91"/>
+      <c r="C5" s="67"/>
       <c r="D5" s="28" t="s">
         <v>100</v>
       </c>
@@ -4807,7 +4807,7 @@
       <c r="B40" t="s">
         <v>105</v>
       </c>
-      <c r="D40" s="144">
+      <c r="D40" s="57">
         <v>0</v>
       </c>
       <c r="H40" s="2">
@@ -4867,123 +4867,123 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:20" ht="72.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B1" s="93" t="s">
+      <c r="B1" s="120" t="s">
         <v>18</v>
       </c>
-      <c r="C1" s="93"/>
-      <c r="D1" s="93"/>
-      <c r="E1" s="93"/>
-      <c r="F1" s="93"/>
-      <c r="G1" s="93"/>
-      <c r="H1" s="93"/>
-      <c r="I1" s="93"/>
-      <c r="J1" s="93"/>
-      <c r="K1" s="93"/>
-      <c r="L1" s="93"/>
-      <c r="M1" s="93"/>
-      <c r="N1" s="93"/>
-      <c r="O1" s="93"/>
-      <c r="P1" s="93"/>
-      <c r="Q1" s="93"/>
-      <c r="R1" s="93"/>
-      <c r="S1" s="93"/>
-      <c r="T1" s="93"/>
+      <c r="C1" s="120"/>
+      <c r="D1" s="120"/>
+      <c r="E1" s="120"/>
+      <c r="F1" s="120"/>
+      <c r="G1" s="120"/>
+      <c r="H1" s="120"/>
+      <c r="I1" s="120"/>
+      <c r="J1" s="120"/>
+      <c r="K1" s="120"/>
+      <c r="L1" s="120"/>
+      <c r="M1" s="120"/>
+      <c r="N1" s="120"/>
+      <c r="O1" s="120"/>
+      <c r="P1" s="120"/>
+      <c r="Q1" s="120"/>
+      <c r="R1" s="120"/>
+      <c r="S1" s="120"/>
+      <c r="T1" s="120"/>
     </row>
     <row r="2" spans="1:20" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A2" s="130" t="s">
+      <c r="A2" s="106" t="s">
         <v>13</v>
       </c>
-      <c r="B2" s="89" t="s">
+      <c r="B2" s="90" t="s">
         <v>21</v>
       </c>
-      <c r="C2" s="65" t="s">
+      <c r="C2" s="66" t="s">
         <v>3</v>
       </c>
-      <c r="D2" s="121" t="str">
+      <c r="D2" s="94" t="str">
         <f>Asistencia!D2</f>
         <v>NOMBRE DOCENTE</v>
       </c>
-      <c r="E2" s="122"/>
-      <c r="F2" s="123"/>
-      <c r="G2" s="121" t="str">
+      <c r="E2" s="95"/>
+      <c r="F2" s="96"/>
+      <c r="G2" s="94" t="str">
         <f>Asistencia!I2</f>
         <v>NOMBRE DOCENTE</v>
       </c>
-      <c r="H2" s="122"/>
-      <c r="I2" s="122"/>
-      <c r="J2" s="122"/>
-      <c r="K2" s="123"/>
-      <c r="L2" s="121" t="s">
+      <c r="H2" s="95"/>
+      <c r="I2" s="95"/>
+      <c r="J2" s="95"/>
+      <c r="K2" s="96"/>
+      <c r="L2" s="94" t="s">
         <v>19</v>
       </c>
-      <c r="M2" s="122"/>
-      <c r="N2" s="122"/>
-      <c r="O2" s="122"/>
-      <c r="P2" s="123"/>
-      <c r="Q2" s="121" t="str">
+      <c r="M2" s="95"/>
+      <c r="N2" s="95"/>
+      <c r="O2" s="95"/>
+      <c r="P2" s="96"/>
+      <c r="Q2" s="94" t="str">
         <f>Asistencia!AA2</f>
         <v>NOMBRE DOCENTE</v>
       </c>
-      <c r="R2" s="122"/>
-      <c r="S2" s="122"/>
-      <c r="T2" s="123"/>
+      <c r="R2" s="95"/>
+      <c r="S2" s="95"/>
+      <c r="T2" s="96"/>
     </row>
     <row r="3" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="131"/>
-      <c r="B3" s="90"/>
-      <c r="C3" s="66"/>
-      <c r="D3" s="138" t="s">
+      <c r="A3" s="107"/>
+      <c r="B3" s="91"/>
+      <c r="C3" s="67"/>
+      <c r="D3" s="114" t="s">
         <v>7</v>
       </c>
-      <c r="E3" s="139"/>
-      <c r="F3" s="140"/>
-      <c r="G3" s="132" t="s">
+      <c r="E3" s="115"/>
+      <c r="F3" s="116"/>
+      <c r="G3" s="108" t="s">
         <v>2</v>
       </c>
-      <c r="H3" s="133"/>
-      <c r="I3" s="133"/>
-      <c r="J3" s="133"/>
-      <c r="K3" s="134"/>
-      <c r="L3" s="115" t="s">
+      <c r="H3" s="109"/>
+      <c r="I3" s="109"/>
+      <c r="J3" s="109"/>
+      <c r="K3" s="110"/>
+      <c r="L3" s="139" t="s">
         <v>1</v>
       </c>
-      <c r="M3" s="116"/>
-      <c r="N3" s="116"/>
-      <c r="O3" s="116"/>
-      <c r="P3" s="117"/>
-      <c r="Q3" s="124" t="s">
-        <v>0</v>
-      </c>
-      <c r="R3" s="125"/>
-      <c r="S3" s="125"/>
-      <c r="T3" s="126"/>
+      <c r="M3" s="140"/>
+      <c r="N3" s="140"/>
+      <c r="O3" s="140"/>
+      <c r="P3" s="141"/>
+      <c r="Q3" s="97" t="s">
+        <v>0</v>
+      </c>
+      <c r="R3" s="98"/>
+      <c r="S3" s="98"/>
+      <c r="T3" s="99"/>
     </row>
     <row r="4" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="131"/>
-      <c r="B4" s="90"/>
-      <c r="C4" s="66"/>
-      <c r="D4" s="141"/>
-      <c r="E4" s="142"/>
-      <c r="F4" s="143"/>
-      <c r="G4" s="135"/>
-      <c r="H4" s="136"/>
-      <c r="I4" s="136"/>
-      <c r="J4" s="136"/>
-      <c r="K4" s="137"/>
-      <c r="L4" s="118"/>
-      <c r="M4" s="119"/>
-      <c r="N4" s="119"/>
-      <c r="O4" s="119"/>
-      <c r="P4" s="120"/>
-      <c r="Q4" s="127"/>
-      <c r="R4" s="128"/>
-      <c r="S4" s="128"/>
-      <c r="T4" s="129"/>
+      <c r="A4" s="107"/>
+      <c r="B4" s="91"/>
+      <c r="C4" s="67"/>
+      <c r="D4" s="117"/>
+      <c r="E4" s="118"/>
+      <c r="F4" s="119"/>
+      <c r="G4" s="111"/>
+      <c r="H4" s="112"/>
+      <c r="I4" s="112"/>
+      <c r="J4" s="112"/>
+      <c r="K4" s="113"/>
+      <c r="L4" s="142"/>
+      <c r="M4" s="143"/>
+      <c r="N4" s="143"/>
+      <c r="O4" s="143"/>
+      <c r="P4" s="144"/>
+      <c r="Q4" s="100"/>
+      <c r="R4" s="101"/>
+      <c r="S4" s="101"/>
+      <c r="T4" s="102"/>
     </row>
     <row r="5" spans="1:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="131"/>
-      <c r="B5" s="90"/>
-      <c r="C5" s="66"/>
+      <c r="A5" s="107"/>
+      <c r="B5" s="91"/>
+      <c r="C5" s="67"/>
       <c r="D5" s="17">
         <v>0.75</v>
       </c>
@@ -6357,12 +6357,14 @@
         <v>0</v>
       </c>
       <c r="G37" s="6"/>
-      <c r="H37" s="6"/>
+      <c r="H37" s="6">
+        <v>3.7</v>
+      </c>
       <c r="I37" s="6"/>
       <c r="J37" s="6"/>
       <c r="K37" s="27">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>0.92500000000000004</v>
       </c>
       <c r="L37" s="6"/>
       <c r="M37" s="6"/>
@@ -7557,195 +7559,186 @@
       </c>
     </row>
     <row r="66" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="D66" s="97" t="s">
+      <c r="D66" s="124" t="s">
         <v>24</v>
       </c>
-      <c r="E66" s="100" t="s">
+      <c r="E66" s="127" t="s">
         <v>12</v>
       </c>
-      <c r="G66" s="94" t="s">
+      <c r="G66" s="121" t="s">
         <v>8</v>
       </c>
-      <c r="H66" s="109" t="s">
+      <c r="H66" s="133" t="s">
         <v>9</v>
       </c>
-      <c r="I66" s="109" t="s">
+      <c r="I66" s="133" t="s">
         <v>10</v>
       </c>
-      <c r="J66" s="94" t="s">
+      <c r="J66" s="121" t="s">
         <v>11</v>
       </c>
       <c r="L66" s="103" t="s">
         <v>8</v>
       </c>
-      <c r="M66" s="106" t="s">
+      <c r="M66" s="130" t="s">
         <v>9</v>
       </c>
-      <c r="N66" s="106" t="s">
+      <c r="N66" s="130" t="s">
         <v>10</v>
       </c>
       <c r="O66" s="103" t="s">
         <v>11</v>
       </c>
-      <c r="Q66" s="112" t="s">
+      <c r="Q66" s="136" t="s">
         <v>24</v>
       </c>
-      <c r="R66" s="112" t="s">
+      <c r="R66" s="136" t="s">
         <v>4</v>
       </c>
-      <c r="S66" s="112" t="s">
+      <c r="S66" s="136" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="67" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="D67" s="98"/>
-      <c r="E67" s="101"/>
-      <c r="G67" s="95"/>
-      <c r="H67" s="110"/>
-      <c r="I67" s="110"/>
-      <c r="J67" s="95"/>
+      <c r="D67" s="125"/>
+      <c r="E67" s="128"/>
+      <c r="G67" s="122"/>
+      <c r="H67" s="134"/>
+      <c r="I67" s="134"/>
+      <c r="J67" s="122"/>
       <c r="L67" s="104"/>
-      <c r="M67" s="107"/>
-      <c r="N67" s="107"/>
+      <c r="M67" s="131"/>
+      <c r="N67" s="131"/>
       <c r="O67" s="104"/>
-      <c r="Q67" s="113"/>
-      <c r="R67" s="113"/>
-      <c r="S67" s="113"/>
+      <c r="Q67" s="137"/>
+      <c r="R67" s="137"/>
+      <c r="S67" s="137"/>
     </row>
     <row r="68" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="D68" s="98"/>
-      <c r="E68" s="101"/>
-      <c r="G68" s="95"/>
-      <c r="H68" s="110"/>
-      <c r="I68" s="110"/>
-      <c r="J68" s="95"/>
+      <c r="D68" s="125"/>
+      <c r="E68" s="128"/>
+      <c r="G68" s="122"/>
+      <c r="H68" s="134"/>
+      <c r="I68" s="134"/>
+      <c r="J68" s="122"/>
       <c r="L68" s="104"/>
-      <c r="M68" s="107"/>
-      <c r="N68" s="107"/>
+      <c r="M68" s="131"/>
+      <c r="N68" s="131"/>
       <c r="O68" s="104"/>
-      <c r="Q68" s="113"/>
-      <c r="R68" s="113"/>
-      <c r="S68" s="113"/>
+      <c r="Q68" s="137"/>
+      <c r="R68" s="137"/>
+      <c r="S68" s="137"/>
     </row>
     <row r="69" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="D69" s="98"/>
-      <c r="E69" s="101"/>
-      <c r="G69" s="95"/>
-      <c r="H69" s="110"/>
-      <c r="I69" s="110"/>
-      <c r="J69" s="95"/>
+      <c r="D69" s="125"/>
+      <c r="E69" s="128"/>
+      <c r="G69" s="122"/>
+      <c r="H69" s="134"/>
+      <c r="I69" s="134"/>
+      <c r="J69" s="122"/>
       <c r="L69" s="104"/>
-      <c r="M69" s="107"/>
-      <c r="N69" s="107"/>
+      <c r="M69" s="131"/>
+      <c r="N69" s="131"/>
       <c r="O69" s="104"/>
-      <c r="Q69" s="113"/>
-      <c r="R69" s="113"/>
-      <c r="S69" s="113"/>
+      <c r="Q69" s="137"/>
+      <c r="R69" s="137"/>
+      <c r="S69" s="137"/>
     </row>
     <row r="70" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="D70" s="98"/>
-      <c r="E70" s="101"/>
-      <c r="G70" s="95"/>
-      <c r="H70" s="110"/>
-      <c r="I70" s="110"/>
-      <c r="J70" s="95"/>
+      <c r="D70" s="125"/>
+      <c r="E70" s="128"/>
+      <c r="G70" s="122"/>
+      <c r="H70" s="134"/>
+      <c r="I70" s="134"/>
+      <c r="J70" s="122"/>
       <c r="L70" s="104"/>
-      <c r="M70" s="107"/>
-      <c r="N70" s="107"/>
+      <c r="M70" s="131"/>
+      <c r="N70" s="131"/>
       <c r="O70" s="104"/>
-      <c r="Q70" s="113"/>
-      <c r="R70" s="113"/>
-      <c r="S70" s="113"/>
+      <c r="Q70" s="137"/>
+      <c r="R70" s="137"/>
+      <c r="S70" s="137"/>
     </row>
     <row r="71" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="D71" s="98"/>
-      <c r="E71" s="101"/>
-      <c r="G71" s="95"/>
-      <c r="H71" s="110"/>
-      <c r="I71" s="110"/>
-      <c r="J71" s="95"/>
+      <c r="D71" s="125"/>
+      <c r="E71" s="128"/>
+      <c r="G71" s="122"/>
+      <c r="H71" s="134"/>
+      <c r="I71" s="134"/>
+      <c r="J71" s="122"/>
       <c r="L71" s="104"/>
-      <c r="M71" s="107"/>
-      <c r="N71" s="107"/>
+      <c r="M71" s="131"/>
+      <c r="N71" s="131"/>
       <c r="O71" s="104"/>
-      <c r="Q71" s="113"/>
-      <c r="R71" s="113"/>
-      <c r="S71" s="113"/>
+      <c r="Q71" s="137"/>
+      <c r="R71" s="137"/>
+      <c r="S71" s="137"/>
     </row>
     <row r="72" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="D72" s="98"/>
-      <c r="E72" s="101"/>
-      <c r="G72" s="95"/>
-      <c r="H72" s="110"/>
-      <c r="I72" s="110"/>
-      <c r="J72" s="95"/>
+      <c r="D72" s="125"/>
+      <c r="E72" s="128"/>
+      <c r="G72" s="122"/>
+      <c r="H72" s="134"/>
+      <c r="I72" s="134"/>
+      <c r="J72" s="122"/>
       <c r="L72" s="104"/>
-      <c r="M72" s="107"/>
-      <c r="N72" s="107"/>
+      <c r="M72" s="131"/>
+      <c r="N72" s="131"/>
       <c r="O72" s="104"/>
-      <c r="Q72" s="113"/>
-      <c r="R72" s="113"/>
-      <c r="S72" s="113"/>
+      <c r="Q72" s="137"/>
+      <c r="R72" s="137"/>
+      <c r="S72" s="137"/>
     </row>
     <row r="73" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="D73" s="98"/>
-      <c r="E73" s="101"/>
-      <c r="G73" s="95"/>
-      <c r="H73" s="110"/>
-      <c r="I73" s="110"/>
-      <c r="J73" s="95"/>
+      <c r="D73" s="125"/>
+      <c r="E73" s="128"/>
+      <c r="G73" s="122"/>
+      <c r="H73" s="134"/>
+      <c r="I73" s="134"/>
+      <c r="J73" s="122"/>
       <c r="L73" s="104"/>
-      <c r="M73" s="107"/>
-      <c r="N73" s="107"/>
+      <c r="M73" s="131"/>
+      <c r="N73" s="131"/>
       <c r="O73" s="104"/>
-      <c r="Q73" s="113"/>
-      <c r="R73" s="113"/>
-      <c r="S73" s="113"/>
+      <c r="Q73" s="137"/>
+      <c r="R73" s="137"/>
+      <c r="S73" s="137"/>
     </row>
     <row r="74" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="D74" s="98"/>
-      <c r="E74" s="101"/>
-      <c r="G74" s="95"/>
-      <c r="H74" s="110"/>
-      <c r="I74" s="110"/>
-      <c r="J74" s="95"/>
+      <c r="D74" s="125"/>
+      <c r="E74" s="128"/>
+      <c r="G74" s="122"/>
+      <c r="H74" s="134"/>
+      <c r="I74" s="134"/>
+      <c r="J74" s="122"/>
       <c r="L74" s="104"/>
-      <c r="M74" s="107"/>
-      <c r="N74" s="107"/>
+      <c r="M74" s="131"/>
+      <c r="N74" s="131"/>
       <c r="O74" s="104"/>
-      <c r="Q74" s="113"/>
-      <c r="R74" s="113"/>
-      <c r="S74" s="113"/>
+      <c r="Q74" s="137"/>
+      <c r="R74" s="137"/>
+      <c r="S74" s="137"/>
     </row>
     <row r="75" spans="1:20" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="D75" s="99"/>
-      <c r="E75" s="102"/>
-      <c r="G75" s="96"/>
-      <c r="H75" s="111"/>
-      <c r="I75" s="111"/>
-      <c r="J75" s="96"/>
+      <c r="D75" s="126"/>
+      <c r="E75" s="129"/>
+      <c r="G75" s="123"/>
+      <c r="H75" s="135"/>
+      <c r="I75" s="135"/>
+      <c r="J75" s="123"/>
       <c r="L75" s="105"/>
-      <c r="M75" s="108"/>
-      <c r="N75" s="108"/>
+      <c r="M75" s="132"/>
+      <c r="N75" s="132"/>
       <c r="O75" s="105"/>
-      <c r="Q75" s="114"/>
-      <c r="R75" s="114"/>
-      <c r="S75" s="114"/>
+      <c r="Q75" s="138"/>
+      <c r="R75" s="138"/>
+      <c r="S75" s="138"/>
     </row>
   </sheetData>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B6:T60">
     <sortCondition ref="B6"/>
   </sortState>
   <mergeCells count="25">
-    <mergeCell ref="G2:K2"/>
-    <mergeCell ref="D2:F2"/>
-    <mergeCell ref="Q3:T4"/>
-    <mergeCell ref="O66:O75"/>
-    <mergeCell ref="A2:A5"/>
-    <mergeCell ref="G3:K4"/>
-    <mergeCell ref="D3:F4"/>
-    <mergeCell ref="B2:B5"/>
-    <mergeCell ref="C2:C5"/>
     <mergeCell ref="B1:T1"/>
     <mergeCell ref="J66:J75"/>
     <mergeCell ref="D66:D75"/>
@@ -7762,6 +7755,15 @@
     <mergeCell ref="I66:I75"/>
     <mergeCell ref="Q2:T2"/>
     <mergeCell ref="L2:P2"/>
+    <mergeCell ref="G2:K2"/>
+    <mergeCell ref="D2:F2"/>
+    <mergeCell ref="Q3:T4"/>
+    <mergeCell ref="O66:O75"/>
+    <mergeCell ref="A2:A5"/>
+    <mergeCell ref="G3:K4"/>
+    <mergeCell ref="D3:F4"/>
+    <mergeCell ref="B2:B5"/>
+    <mergeCell ref="C2:C5"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
mejor forma para resolver problema de los ciclístas.
</commit_message>
<xml_diff>
--- a/9_asistencia_evaluacion/pivu_caucasia.xlsx
+++ b/9_asistencia_evaluacion/pivu_caucasia.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\marco\Documentos\extension\camino-udea\9_asistencia_evaluacion\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{05C23E8C-083C-4F68-9B5D-1FBD65DA9124}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{70D4DA88-E0DF-4EB6-93CF-45B1295C9DB5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1028,6 +1028,192 @@
     <xf numFmtId="0" fontId="12" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="19" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="7" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="8" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="9" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="9" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="9" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="6" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="11" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="11" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1058,15 +1244,6 @@
     <xf numFmtId="0" fontId="7" fillId="6" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="9" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
     </xf>
@@ -1110,183 +1287,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="9" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="11" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="11" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="7" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="8" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="9" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="9" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="9" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="9" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="9" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="9" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="6" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1786,28 +1786,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="72" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="114" t="s">
+      <c r="A1" s="93" t="s">
         <v>27</v>
       </c>
-      <c r="B1" s="113"/>
-      <c r="C1" s="113"/>
-      <c r="D1" s="113"/>
-      <c r="E1" s="113"/>
-      <c r="F1" s="113"/>
-      <c r="G1" s="113"/>
-      <c r="H1" s="113"/>
+      <c r="B1" s="92"/>
+      <c r="C1" s="92"/>
+      <c r="D1" s="92"/>
+      <c r="E1" s="92"/>
+      <c r="F1" s="92"/>
+      <c r="G1" s="92"/>
+      <c r="H1" s="92"/>
     </row>
     <row r="2" spans="1:9" ht="19.8" x14ac:dyDescent="0.3">
-      <c r="A2" s="113" t="s">
+      <c r="A2" s="92" t="s">
         <v>26</v>
       </c>
-      <c r="B2" s="113"/>
-      <c r="C2" s="113"/>
-      <c r="D2" s="113"/>
-      <c r="E2" s="113"/>
-      <c r="F2" s="113"/>
-      <c r="G2" s="113"/>
-      <c r="H2" s="113"/>
+      <c r="B2" s="92"/>
+      <c r="C2" s="92"/>
+      <c r="D2" s="92"/>
+      <c r="E2" s="92"/>
+      <c r="F2" s="92"/>
+      <c r="G2" s="92"/>
+      <c r="H2" s="92"/>
       <c r="I2" s="50" t="s">
         <v>99</v>
       </c>
@@ -2729,172 +2729,172 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:31" ht="66" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B1" s="122" t="s">
+      <c r="B1" s="65" t="s">
         <v>18</v>
       </c>
-      <c r="C1" s="122"/>
-      <c r="D1" s="122"/>
-      <c r="E1" s="122"/>
-      <c r="F1" s="122"/>
-      <c r="G1" s="122"/>
-      <c r="H1" s="122"/>
-      <c r="I1" s="122"/>
-      <c r="J1" s="122"/>
-      <c r="K1" s="122"/>
-      <c r="L1" s="122"/>
-      <c r="M1" s="122"/>
-      <c r="N1" s="122"/>
-      <c r="O1" s="122"/>
-      <c r="P1" s="122"/>
-      <c r="Q1" s="122"/>
-      <c r="R1" s="122"/>
-      <c r="S1" s="122"/>
-      <c r="T1" s="122"/>
-      <c r="U1" s="122"/>
-      <c r="V1" s="122"/>
-      <c r="W1" s="122"/>
-      <c r="X1" s="122"/>
-      <c r="Y1" s="122"/>
-      <c r="Z1" s="122"/>
-      <c r="AA1" s="122"/>
-      <c r="AB1" s="122"/>
-      <c r="AC1" s="122"/>
-      <c r="AD1" s="122"/>
-      <c r="AE1" s="122"/>
+      <c r="C1" s="65"/>
+      <c r="D1" s="65"/>
+      <c r="E1" s="65"/>
+      <c r="F1" s="65"/>
+      <c r="G1" s="65"/>
+      <c r="H1" s="65"/>
+      <c r="I1" s="65"/>
+      <c r="J1" s="65"/>
+      <c r="K1" s="65"/>
+      <c r="L1" s="65"/>
+      <c r="M1" s="65"/>
+      <c r="N1" s="65"/>
+      <c r="O1" s="65"/>
+      <c r="P1" s="65"/>
+      <c r="Q1" s="65"/>
+      <c r="R1" s="65"/>
+      <c r="S1" s="65"/>
+      <c r="T1" s="65"/>
+      <c r="U1" s="65"/>
+      <c r="V1" s="65"/>
+      <c r="W1" s="65"/>
+      <c r="X1" s="65"/>
+      <c r="Y1" s="65"/>
+      <c r="Z1" s="65"/>
+      <c r="AA1" s="65"/>
+      <c r="AB1" s="65"/>
+      <c r="AC1" s="65"/>
+      <c r="AD1" s="65"/>
+      <c r="AE1" s="65"/>
     </row>
     <row r="2" spans="1:31" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A2" s="111" t="s">
+      <c r="A2" s="66" t="s">
         <v>13</v>
       </c>
-      <c r="B2" s="109" t="s">
+      <c r="B2" s="90" t="s">
         <v>21</v>
       </c>
-      <c r="C2" s="111" t="s">
+      <c r="C2" s="66" t="s">
         <v>3</v>
       </c>
-      <c r="D2" s="138" t="s">
+      <c r="D2" s="83" t="s">
         <v>19</v>
       </c>
-      <c r="E2" s="139"/>
-      <c r="F2" s="139"/>
-      <c r="G2" s="139"/>
-      <c r="H2" s="140"/>
-      <c r="I2" s="123" t="s">
+      <c r="E2" s="84"/>
+      <c r="F2" s="84"/>
+      <c r="G2" s="84"/>
+      <c r="H2" s="85"/>
+      <c r="I2" s="68" t="s">
         <v>19</v>
       </c>
-      <c r="J2" s="124"/>
-      <c r="K2" s="124"/>
-      <c r="L2" s="124"/>
-      <c r="M2" s="124"/>
-      <c r="N2" s="124"/>
-      <c r="O2" s="124"/>
-      <c r="P2" s="124"/>
-      <c r="Q2" s="125"/>
-      <c r="R2" s="132" t="s">
+      <c r="J2" s="69"/>
+      <c r="K2" s="69"/>
+      <c r="L2" s="69"/>
+      <c r="M2" s="69"/>
+      <c r="N2" s="69"/>
+      <c r="O2" s="69"/>
+      <c r="P2" s="69"/>
+      <c r="Q2" s="70"/>
+      <c r="R2" s="77" t="s">
         <v>19</v>
       </c>
-      <c r="S2" s="133"/>
-      <c r="T2" s="133"/>
-      <c r="U2" s="133"/>
-      <c r="V2" s="133"/>
-      <c r="W2" s="133"/>
-      <c r="X2" s="133"/>
-      <c r="Y2" s="133"/>
-      <c r="Z2" s="134"/>
-      <c r="AA2" s="115" t="s">
+      <c r="S2" s="78"/>
+      <c r="T2" s="78"/>
+      <c r="U2" s="78"/>
+      <c r="V2" s="78"/>
+      <c r="W2" s="78"/>
+      <c r="X2" s="78"/>
+      <c r="Y2" s="78"/>
+      <c r="Z2" s="79"/>
+      <c r="AA2" s="58" t="s">
         <v>19</v>
       </c>
-      <c r="AB2" s="116"/>
-      <c r="AC2" s="116"/>
-      <c r="AD2" s="116"/>
-      <c r="AE2" s="117"/>
+      <c r="AB2" s="59"/>
+      <c r="AC2" s="59"/>
+      <c r="AD2" s="59"/>
+      <c r="AE2" s="60"/>
     </row>
     <row r="3" spans="1:31" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="112"/>
-      <c r="B3" s="110"/>
-      <c r="C3" s="112"/>
-      <c r="D3" s="141" t="s">
+      <c r="A3" s="67"/>
+      <c r="B3" s="91"/>
+      <c r="C3" s="67"/>
+      <c r="D3" s="86" t="s">
         <v>7</v>
       </c>
-      <c r="E3" s="142"/>
-      <c r="F3" s="142"/>
-      <c r="G3" s="142"/>
-      <c r="H3" s="143"/>
-      <c r="I3" s="126" t="s">
+      <c r="E3" s="87"/>
+      <c r="F3" s="87"/>
+      <c r="G3" s="87"/>
+      <c r="H3" s="88"/>
+      <c r="I3" s="71" t="s">
         <v>2</v>
       </c>
-      <c r="J3" s="127"/>
-      <c r="K3" s="127"/>
-      <c r="L3" s="127"/>
-      <c r="M3" s="127"/>
-      <c r="N3" s="127"/>
-      <c r="O3" s="127"/>
-      <c r="P3" s="127"/>
-      <c r="Q3" s="128"/>
-      <c r="R3" s="135" t="s">
+      <c r="J3" s="72"/>
+      <c r="K3" s="72"/>
+      <c r="L3" s="72"/>
+      <c r="M3" s="72"/>
+      <c r="N3" s="72"/>
+      <c r="O3" s="72"/>
+      <c r="P3" s="72"/>
+      <c r="Q3" s="73"/>
+      <c r="R3" s="80" t="s">
         <v>1</v>
       </c>
-      <c r="S3" s="136"/>
-      <c r="T3" s="136"/>
-      <c r="U3" s="136"/>
-      <c r="V3" s="136"/>
-      <c r="W3" s="136"/>
-      <c r="X3" s="136"/>
-      <c r="Y3" s="136"/>
-      <c r="Z3" s="137"/>
-      <c r="AA3" s="118" t="s">
-        <v>0</v>
-      </c>
-      <c r="AB3" s="119"/>
-      <c r="AC3" s="119"/>
-      <c r="AD3" s="119"/>
-      <c r="AE3" s="120"/>
+      <c r="S3" s="81"/>
+      <c r="T3" s="81"/>
+      <c r="U3" s="81"/>
+      <c r="V3" s="81"/>
+      <c r="W3" s="81"/>
+      <c r="X3" s="81"/>
+      <c r="Y3" s="81"/>
+      <c r="Z3" s="82"/>
+      <c r="AA3" s="61" t="s">
+        <v>0</v>
+      </c>
+      <c r="AB3" s="62"/>
+      <c r="AC3" s="62"/>
+      <c r="AD3" s="62"/>
+      <c r="AE3" s="63"/>
     </row>
     <row r="4" spans="1:31" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="112"/>
-      <c r="B4" s="110"/>
-      <c r="C4" s="112"/>
-      <c r="D4" s="144" t="s">
+      <c r="A4" s="67"/>
+      <c r="B4" s="91"/>
+      <c r="C4" s="67"/>
+      <c r="D4" s="89" t="s">
         <v>22</v>
       </c>
-      <c r="E4" s="130"/>
-      <c r="F4" s="130"/>
-      <c r="G4" s="131"/>
+      <c r="E4" s="75"/>
+      <c r="F4" s="75"/>
+      <c r="G4" s="76"/>
       <c r="H4" s="1"/>
-      <c r="I4" s="129" t="s">
+      <c r="I4" s="74" t="s">
         <v>23</v>
       </c>
-      <c r="J4" s="130"/>
-      <c r="K4" s="130"/>
-      <c r="L4" s="130"/>
-      <c r="M4" s="130"/>
-      <c r="N4" s="130"/>
-      <c r="O4" s="130"/>
-      <c r="P4" s="131"/>
+      <c r="J4" s="75"/>
+      <c r="K4" s="75"/>
+      <c r="L4" s="75"/>
+      <c r="M4" s="75"/>
+      <c r="N4" s="75"/>
+      <c r="O4" s="75"/>
+      <c r="P4" s="76"/>
       <c r="Q4" s="3"/>
-      <c r="R4" s="129" t="s">
+      <c r="R4" s="74" t="s">
         <v>23</v>
       </c>
-      <c r="S4" s="130"/>
-      <c r="T4" s="130"/>
-      <c r="U4" s="130"/>
-      <c r="V4" s="130"/>
-      <c r="W4" s="130"/>
-      <c r="X4" s="130"/>
-      <c r="Y4" s="131"/>
+      <c r="S4" s="75"/>
+      <c r="T4" s="75"/>
+      <c r="U4" s="75"/>
+      <c r="V4" s="75"/>
+      <c r="W4" s="75"/>
+      <c r="X4" s="75"/>
+      <c r="Y4" s="76"/>
       <c r="Z4" s="12"/>
-      <c r="AA4" s="121" t="s">
+      <c r="AA4" s="64" t="s">
         <v>23</v>
       </c>
-      <c r="AB4" s="121"/>
-      <c r="AC4" s="121"/>
-      <c r="AD4" s="121"/>
+      <c r="AB4" s="64"/>
+      <c r="AC4" s="64"/>
+      <c r="AD4" s="64"/>
       <c r="AE4" s="3"/>
     </row>
     <row r="5" spans="1:31" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="112"/>
-      <c r="B5" s="110"/>
-      <c r="C5" s="112"/>
+      <c r="A5" s="67"/>
+      <c r="B5" s="91"/>
+      <c r="C5" s="67"/>
       <c r="D5" s="28" t="s">
         <v>100</v>
       </c>
@@ -3002,14 +3002,14 @@
         <v>1038117202</v>
       </c>
       <c r="D7" s="13">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E7" s="13"/>
       <c r="F7" s="13"/>
       <c r="G7" s="13"/>
       <c r="H7" s="32">
         <f t="shared" ref="H7:H40" si="0">+SUM(D7:G7)/4</f>
-        <v>0.25</v>
+        <v>0.5</v>
       </c>
       <c r="I7" s="33"/>
       <c r="J7" s="33"/>
@@ -3057,14 +3057,14 @@
         <v>1041633525</v>
       </c>
       <c r="D8" s="13">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E8" s="13"/>
       <c r="F8" s="13"/>
       <c r="G8" s="13"/>
       <c r="H8" s="32">
         <f t="shared" si="0"/>
-        <v>1</v>
+        <v>1.25</v>
       </c>
       <c r="I8" s="33"/>
       <c r="J8" s="33"/>
@@ -3222,14 +3222,14 @@
         <v>1038110143</v>
       </c>
       <c r="D11" s="13">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E11" s="13"/>
       <c r="F11" s="13"/>
       <c r="G11" s="13"/>
       <c r="H11" s="32">
         <f t="shared" si="0"/>
-        <v>0.75</v>
+        <v>1</v>
       </c>
       <c r="I11" s="33"/>
       <c r="J11" s="33"/>
@@ -3387,14 +3387,14 @@
         <v>1038111245</v>
       </c>
       <c r="D14" s="13">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E14" s="13"/>
       <c r="F14" s="13"/>
       <c r="G14" s="13"/>
       <c r="H14" s="32">
         <f t="shared" si="0"/>
-        <v>1.75</v>
+        <v>2</v>
       </c>
       <c r="I14" s="33"/>
       <c r="J14" s="33"/>
@@ -3442,14 +3442,14 @@
         <v>1038134078</v>
       </c>
       <c r="D15" s="13">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E15" s="13"/>
       <c r="F15" s="13"/>
       <c r="G15" s="13"/>
       <c r="H15" s="32">
         <f t="shared" si="0"/>
-        <v>0.5</v>
+        <v>0.75</v>
       </c>
       <c r="I15" s="33"/>
       <c r="J15" s="33"/>
@@ -3717,14 +3717,14 @@
         <v>1038105559</v>
       </c>
       <c r="D20" s="13">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E20" s="13"/>
       <c r="F20" s="13"/>
       <c r="G20" s="13"/>
       <c r="H20" s="32">
         <f t="shared" si="0"/>
-        <v>1</v>
+        <v>1.25</v>
       </c>
       <c r="I20" s="33"/>
       <c r="J20" s="33"/>
@@ -3827,14 +3827,14 @@
         <v>1038114154</v>
       </c>
       <c r="D22" s="13">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E22" s="13"/>
       <c r="F22" s="13"/>
       <c r="G22" s="13"/>
       <c r="H22" s="32">
         <f t="shared" si="0"/>
-        <v>0.25</v>
+        <v>0</v>
       </c>
       <c r="I22" s="33"/>
       <c r="J22" s="33"/>
@@ -3882,14 +3882,14 @@
         <v>1038113598</v>
       </c>
       <c r="D23" s="13">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E23" s="13"/>
       <c r="F23" s="13"/>
       <c r="G23" s="13"/>
       <c r="H23" s="32">
         <f t="shared" si="0"/>
-        <v>0.25</v>
+        <v>0.5</v>
       </c>
       <c r="I23" s="33"/>
       <c r="J23" s="33"/>
@@ -3936,13 +3936,15 @@
         <f>+Inscritos!D22</f>
         <v>1038648337</v>
       </c>
-      <c r="D24" s="13"/>
+      <c r="D24" s="13">
+        <v>1</v>
+      </c>
       <c r="E24" s="13"/>
       <c r="F24" s="13"/>
       <c r="G24" s="13"/>
       <c r="H24" s="32">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>0.25</v>
       </c>
       <c r="I24" s="33"/>
       <c r="J24" s="33"/>
@@ -4153,14 +4155,14 @@
         <v>1038115554</v>
       </c>
       <c r="D28" s="13">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E28" s="13"/>
       <c r="F28" s="13"/>
       <c r="G28" s="13"/>
       <c r="H28" s="32">
         <f t="shared" si="0"/>
-        <v>0.25</v>
+        <v>0.5</v>
       </c>
       <c r="I28" s="33"/>
       <c r="J28" s="33"/>
@@ -4373,14 +4375,14 @@
         <v>1038104210</v>
       </c>
       <c r="D32" s="13">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E32" s="13"/>
       <c r="F32" s="13"/>
       <c r="G32" s="13"/>
       <c r="H32" s="32">
         <f t="shared" si="0"/>
-        <v>2</v>
+        <v>2.25</v>
       </c>
       <c r="I32" s="33"/>
       <c r="J32" s="33"/>
@@ -4483,14 +4485,14 @@
         <v>1038111917</v>
       </c>
       <c r="D34" s="13">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E34" s="13"/>
       <c r="F34" s="13"/>
       <c r="G34" s="13"/>
       <c r="H34" s="32">
         <f t="shared" si="0"/>
-        <v>0.25</v>
+        <v>0</v>
       </c>
       <c r="I34" s="33"/>
       <c r="J34" s="33"/>
@@ -4538,14 +4540,14 @@
         <v>1038115337</v>
       </c>
       <c r="D35" s="13">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E35" s="13"/>
       <c r="F35" s="13"/>
       <c r="G35" s="13"/>
       <c r="H35" s="32">
         <f t="shared" si="0"/>
-        <v>1</v>
+        <v>1.25</v>
       </c>
       <c r="I35" s="33"/>
       <c r="J35" s="33"/>
@@ -4593,14 +4595,14 @@
         <v>1116074065</v>
       </c>
       <c r="D36" s="13">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E36" s="13"/>
       <c r="F36" s="13"/>
       <c r="G36" s="13"/>
       <c r="H36" s="32">
         <f t="shared" si="0"/>
-        <v>0.5</v>
+        <v>0.75</v>
       </c>
       <c r="I36" s="33"/>
       <c r="J36" s="33"/>
@@ -4758,14 +4760,14 @@
         <v>1038113397</v>
       </c>
       <c r="D39" s="13">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E39" s="13"/>
       <c r="F39" s="13"/>
       <c r="G39" s="13"/>
       <c r="H39" s="32">
         <f t="shared" si="0"/>
-        <v>0.5</v>
+        <v>0.75</v>
       </c>
       <c r="I39" s="33"/>
       <c r="J39" s="33"/>
@@ -4867,123 +4869,123 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:20" ht="72.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B1" s="58" t="s">
+      <c r="B1" s="120" t="s">
         <v>18</v>
       </c>
-      <c r="C1" s="58"/>
-      <c r="D1" s="58"/>
-      <c r="E1" s="58"/>
-      <c r="F1" s="58"/>
-      <c r="G1" s="58"/>
-      <c r="H1" s="58"/>
-      <c r="I1" s="58"/>
-      <c r="J1" s="58"/>
-      <c r="K1" s="58"/>
-      <c r="L1" s="58"/>
-      <c r="M1" s="58"/>
-      <c r="N1" s="58"/>
-      <c r="O1" s="58"/>
-      <c r="P1" s="58"/>
-      <c r="Q1" s="58"/>
-      <c r="R1" s="58"/>
-      <c r="S1" s="58"/>
-      <c r="T1" s="58"/>
+      <c r="C1" s="120"/>
+      <c r="D1" s="120"/>
+      <c r="E1" s="120"/>
+      <c r="F1" s="120"/>
+      <c r="G1" s="120"/>
+      <c r="H1" s="120"/>
+      <c r="I1" s="120"/>
+      <c r="J1" s="120"/>
+      <c r="K1" s="120"/>
+      <c r="L1" s="120"/>
+      <c r="M1" s="120"/>
+      <c r="N1" s="120"/>
+      <c r="O1" s="120"/>
+      <c r="P1" s="120"/>
+      <c r="Q1" s="120"/>
+      <c r="R1" s="120"/>
+      <c r="S1" s="120"/>
+      <c r="T1" s="120"/>
     </row>
     <row r="2" spans="1:20" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A2" s="95" t="s">
+      <c r="A2" s="106" t="s">
         <v>13</v>
       </c>
-      <c r="B2" s="109" t="s">
+      <c r="B2" s="90" t="s">
         <v>21</v>
       </c>
-      <c r="C2" s="111" t="s">
+      <c r="C2" s="66" t="s">
         <v>3</v>
       </c>
-      <c r="D2" s="86" t="str">
+      <c r="D2" s="94" t="str">
         <f>Asistencia!D2</f>
         <v>NOMBRE DOCENTE</v>
       </c>
-      <c r="E2" s="87"/>
-      <c r="F2" s="88"/>
-      <c r="G2" s="86" t="str">
+      <c r="E2" s="95"/>
+      <c r="F2" s="96"/>
+      <c r="G2" s="94" t="str">
         <f>Asistencia!I2</f>
         <v>NOMBRE DOCENTE</v>
       </c>
-      <c r="H2" s="87"/>
-      <c r="I2" s="87"/>
-      <c r="J2" s="87"/>
-      <c r="K2" s="88"/>
-      <c r="L2" s="86" t="s">
+      <c r="H2" s="95"/>
+      <c r="I2" s="95"/>
+      <c r="J2" s="95"/>
+      <c r="K2" s="96"/>
+      <c r="L2" s="94" t="s">
         <v>19</v>
       </c>
-      <c r="M2" s="87"/>
-      <c r="N2" s="87"/>
-      <c r="O2" s="87"/>
-      <c r="P2" s="88"/>
-      <c r="Q2" s="86" t="str">
+      <c r="M2" s="95"/>
+      <c r="N2" s="95"/>
+      <c r="O2" s="95"/>
+      <c r="P2" s="96"/>
+      <c r="Q2" s="94" t="str">
         <f>Asistencia!AA2</f>
         <v>NOMBRE DOCENTE</v>
       </c>
-      <c r="R2" s="87"/>
-      <c r="S2" s="87"/>
-      <c r="T2" s="88"/>
+      <c r="R2" s="95"/>
+      <c r="S2" s="95"/>
+      <c r="T2" s="96"/>
     </row>
     <row r="3" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="96"/>
-      <c r="B3" s="110"/>
-      <c r="C3" s="112"/>
-      <c r="D3" s="103" t="s">
+      <c r="A3" s="107"/>
+      <c r="B3" s="91"/>
+      <c r="C3" s="67"/>
+      <c r="D3" s="114" t="s">
         <v>7</v>
       </c>
-      <c r="E3" s="104"/>
-      <c r="F3" s="105"/>
-      <c r="G3" s="97" t="s">
+      <c r="E3" s="115"/>
+      <c r="F3" s="116"/>
+      <c r="G3" s="108" t="s">
         <v>2</v>
       </c>
-      <c r="H3" s="98"/>
-      <c r="I3" s="98"/>
-      <c r="J3" s="98"/>
-      <c r="K3" s="99"/>
-      <c r="L3" s="80" t="s">
+      <c r="H3" s="109"/>
+      <c r="I3" s="109"/>
+      <c r="J3" s="109"/>
+      <c r="K3" s="110"/>
+      <c r="L3" s="139" t="s">
         <v>1</v>
       </c>
-      <c r="M3" s="81"/>
-      <c r="N3" s="81"/>
-      <c r="O3" s="81"/>
-      <c r="P3" s="82"/>
-      <c r="Q3" s="89" t="s">
-        <v>0</v>
-      </c>
-      <c r="R3" s="90"/>
-      <c r="S3" s="90"/>
-      <c r="T3" s="91"/>
+      <c r="M3" s="140"/>
+      <c r="N3" s="140"/>
+      <c r="O3" s="140"/>
+      <c r="P3" s="141"/>
+      <c r="Q3" s="97" t="s">
+        <v>0</v>
+      </c>
+      <c r="R3" s="98"/>
+      <c r="S3" s="98"/>
+      <c r="T3" s="99"/>
     </row>
     <row r="4" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="96"/>
-      <c r="B4" s="110"/>
-      <c r="C4" s="112"/>
-      <c r="D4" s="106"/>
-      <c r="E4" s="107"/>
-      <c r="F4" s="108"/>
-      <c r="G4" s="100"/>
-      <c r="H4" s="101"/>
-      <c r="I4" s="101"/>
-      <c r="J4" s="101"/>
-      <c r="K4" s="102"/>
-      <c r="L4" s="83"/>
-      <c r="M4" s="84"/>
-      <c r="N4" s="84"/>
-      <c r="O4" s="84"/>
-      <c r="P4" s="85"/>
-      <c r="Q4" s="92"/>
-      <c r="R4" s="93"/>
-      <c r="S4" s="93"/>
-      <c r="T4" s="94"/>
+      <c r="A4" s="107"/>
+      <c r="B4" s="91"/>
+      <c r="C4" s="67"/>
+      <c r="D4" s="117"/>
+      <c r="E4" s="118"/>
+      <c r="F4" s="119"/>
+      <c r="G4" s="111"/>
+      <c r="H4" s="112"/>
+      <c r="I4" s="112"/>
+      <c r="J4" s="112"/>
+      <c r="K4" s="113"/>
+      <c r="L4" s="142"/>
+      <c r="M4" s="143"/>
+      <c r="N4" s="143"/>
+      <c r="O4" s="143"/>
+      <c r="P4" s="144"/>
+      <c r="Q4" s="100"/>
+      <c r="R4" s="101"/>
+      <c r="S4" s="101"/>
+      <c r="T4" s="102"/>
     </row>
     <row r="5" spans="1:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="96"/>
-      <c r="B5" s="110"/>
-      <c r="C5" s="112"/>
+      <c r="A5" s="107"/>
+      <c r="B5" s="91"/>
+      <c r="C5" s="67"/>
       <c r="D5" s="17">
         <v>0.75</v>
       </c>
@@ -7559,195 +7561,186 @@
       </c>
     </row>
     <row r="66" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="D66" s="62" t="s">
+      <c r="D66" s="124" t="s">
         <v>24</v>
       </c>
-      <c r="E66" s="65" t="s">
+      <c r="E66" s="127" t="s">
         <v>12</v>
       </c>
-      <c r="G66" s="59" t="s">
+      <c r="G66" s="121" t="s">
         <v>8</v>
       </c>
-      <c r="H66" s="74" t="s">
+      <c r="H66" s="133" t="s">
         <v>9</v>
       </c>
-      <c r="I66" s="74" t="s">
+      <c r="I66" s="133" t="s">
         <v>10</v>
       </c>
-      <c r="J66" s="59" t="s">
+      <c r="J66" s="121" t="s">
         <v>11</v>
       </c>
-      <c r="L66" s="68" t="s">
+      <c r="L66" s="103" t="s">
         <v>8</v>
       </c>
-      <c r="M66" s="71" t="s">
+      <c r="M66" s="130" t="s">
         <v>9</v>
       </c>
-      <c r="N66" s="71" t="s">
+      <c r="N66" s="130" t="s">
         <v>10</v>
       </c>
-      <c r="O66" s="68" t="s">
+      <c r="O66" s="103" t="s">
         <v>11</v>
       </c>
-      <c r="Q66" s="77" t="s">
+      <c r="Q66" s="136" t="s">
         <v>24</v>
       </c>
-      <c r="R66" s="77" t="s">
+      <c r="R66" s="136" t="s">
         <v>4</v>
       </c>
-      <c r="S66" s="77" t="s">
+      <c r="S66" s="136" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="67" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="D67" s="63"/>
-      <c r="E67" s="66"/>
-      <c r="G67" s="60"/>
-      <c r="H67" s="75"/>
-      <c r="I67" s="75"/>
-      <c r="J67" s="60"/>
-      <c r="L67" s="69"/>
-      <c r="M67" s="72"/>
-      <c r="N67" s="72"/>
-      <c r="O67" s="69"/>
-      <c r="Q67" s="78"/>
-      <c r="R67" s="78"/>
-      <c r="S67" s="78"/>
+      <c r="D67" s="125"/>
+      <c r="E67" s="128"/>
+      <c r="G67" s="122"/>
+      <c r="H67" s="134"/>
+      <c r="I67" s="134"/>
+      <c r="J67" s="122"/>
+      <c r="L67" s="104"/>
+      <c r="M67" s="131"/>
+      <c r="N67" s="131"/>
+      <c r="O67" s="104"/>
+      <c r="Q67" s="137"/>
+      <c r="R67" s="137"/>
+      <c r="S67" s="137"/>
     </row>
     <row r="68" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="D68" s="63"/>
-      <c r="E68" s="66"/>
-      <c r="G68" s="60"/>
-      <c r="H68" s="75"/>
-      <c r="I68" s="75"/>
-      <c r="J68" s="60"/>
-      <c r="L68" s="69"/>
-      <c r="M68" s="72"/>
-      <c r="N68" s="72"/>
-      <c r="O68" s="69"/>
-      <c r="Q68" s="78"/>
-      <c r="R68" s="78"/>
-      <c r="S68" s="78"/>
+      <c r="D68" s="125"/>
+      <c r="E68" s="128"/>
+      <c r="G68" s="122"/>
+      <c r="H68" s="134"/>
+      <c r="I68" s="134"/>
+      <c r="J68" s="122"/>
+      <c r="L68" s="104"/>
+      <c r="M68" s="131"/>
+      <c r="N68" s="131"/>
+      <c r="O68" s="104"/>
+      <c r="Q68" s="137"/>
+      <c r="R68" s="137"/>
+      <c r="S68" s="137"/>
     </row>
     <row r="69" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="D69" s="63"/>
-      <c r="E69" s="66"/>
-      <c r="G69" s="60"/>
-      <c r="H69" s="75"/>
-      <c r="I69" s="75"/>
-      <c r="J69" s="60"/>
-      <c r="L69" s="69"/>
-      <c r="M69" s="72"/>
-      <c r="N69" s="72"/>
-      <c r="O69" s="69"/>
-      <c r="Q69" s="78"/>
-      <c r="R69" s="78"/>
-      <c r="S69" s="78"/>
+      <c r="D69" s="125"/>
+      <c r="E69" s="128"/>
+      <c r="G69" s="122"/>
+      <c r="H69" s="134"/>
+      <c r="I69" s="134"/>
+      <c r="J69" s="122"/>
+      <c r="L69" s="104"/>
+      <c r="M69" s="131"/>
+      <c r="N69" s="131"/>
+      <c r="O69" s="104"/>
+      <c r="Q69" s="137"/>
+      <c r="R69" s="137"/>
+      <c r="S69" s="137"/>
     </row>
     <row r="70" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="D70" s="63"/>
-      <c r="E70" s="66"/>
-      <c r="G70" s="60"/>
-      <c r="H70" s="75"/>
-      <c r="I70" s="75"/>
-      <c r="J70" s="60"/>
-      <c r="L70" s="69"/>
-      <c r="M70" s="72"/>
-      <c r="N70" s="72"/>
-      <c r="O70" s="69"/>
-      <c r="Q70" s="78"/>
-      <c r="R70" s="78"/>
-      <c r="S70" s="78"/>
+      <c r="D70" s="125"/>
+      <c r="E70" s="128"/>
+      <c r="G70" s="122"/>
+      <c r="H70" s="134"/>
+      <c r="I70" s="134"/>
+      <c r="J70" s="122"/>
+      <c r="L70" s="104"/>
+      <c r="M70" s="131"/>
+      <c r="N70" s="131"/>
+      <c r="O70" s="104"/>
+      <c r="Q70" s="137"/>
+      <c r="R70" s="137"/>
+      <c r="S70" s="137"/>
     </row>
     <row r="71" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="D71" s="63"/>
-      <c r="E71" s="66"/>
-      <c r="G71" s="60"/>
-      <c r="H71" s="75"/>
-      <c r="I71" s="75"/>
-      <c r="J71" s="60"/>
-      <c r="L71" s="69"/>
-      <c r="M71" s="72"/>
-      <c r="N71" s="72"/>
-      <c r="O71" s="69"/>
-      <c r="Q71" s="78"/>
-      <c r="R71" s="78"/>
-      <c r="S71" s="78"/>
+      <c r="D71" s="125"/>
+      <c r="E71" s="128"/>
+      <c r="G71" s="122"/>
+      <c r="H71" s="134"/>
+      <c r="I71" s="134"/>
+      <c r="J71" s="122"/>
+      <c r="L71" s="104"/>
+      <c r="M71" s="131"/>
+      <c r="N71" s="131"/>
+      <c r="O71" s="104"/>
+      <c r="Q71" s="137"/>
+      <c r="R71" s="137"/>
+      <c r="S71" s="137"/>
     </row>
     <row r="72" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="D72" s="63"/>
-      <c r="E72" s="66"/>
-      <c r="G72" s="60"/>
-      <c r="H72" s="75"/>
-      <c r="I72" s="75"/>
-      <c r="J72" s="60"/>
-      <c r="L72" s="69"/>
-      <c r="M72" s="72"/>
-      <c r="N72" s="72"/>
-      <c r="O72" s="69"/>
-      <c r="Q72" s="78"/>
-      <c r="R72" s="78"/>
-      <c r="S72" s="78"/>
+      <c r="D72" s="125"/>
+      <c r="E72" s="128"/>
+      <c r="G72" s="122"/>
+      <c r="H72" s="134"/>
+      <c r="I72" s="134"/>
+      <c r="J72" s="122"/>
+      <c r="L72" s="104"/>
+      <c r="M72" s="131"/>
+      <c r="N72" s="131"/>
+      <c r="O72" s="104"/>
+      <c r="Q72" s="137"/>
+      <c r="R72" s="137"/>
+      <c r="S72" s="137"/>
     </row>
     <row r="73" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="D73" s="63"/>
-      <c r="E73" s="66"/>
-      <c r="G73" s="60"/>
-      <c r="H73" s="75"/>
-      <c r="I73" s="75"/>
-      <c r="J73" s="60"/>
-      <c r="L73" s="69"/>
-      <c r="M73" s="72"/>
-      <c r="N73" s="72"/>
-      <c r="O73" s="69"/>
-      <c r="Q73" s="78"/>
-      <c r="R73" s="78"/>
-      <c r="S73" s="78"/>
+      <c r="D73" s="125"/>
+      <c r="E73" s="128"/>
+      <c r="G73" s="122"/>
+      <c r="H73" s="134"/>
+      <c r="I73" s="134"/>
+      <c r="J73" s="122"/>
+      <c r="L73" s="104"/>
+      <c r="M73" s="131"/>
+      <c r="N73" s="131"/>
+      <c r="O73" s="104"/>
+      <c r="Q73" s="137"/>
+      <c r="R73" s="137"/>
+      <c r="S73" s="137"/>
     </row>
     <row r="74" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="D74" s="63"/>
-      <c r="E74" s="66"/>
-      <c r="G74" s="60"/>
-      <c r="H74" s="75"/>
-      <c r="I74" s="75"/>
-      <c r="J74" s="60"/>
-      <c r="L74" s="69"/>
-      <c r="M74" s="72"/>
-      <c r="N74" s="72"/>
-      <c r="O74" s="69"/>
-      <c r="Q74" s="78"/>
-      <c r="R74" s="78"/>
-      <c r="S74" s="78"/>
+      <c r="D74" s="125"/>
+      <c r="E74" s="128"/>
+      <c r="G74" s="122"/>
+      <c r="H74" s="134"/>
+      <c r="I74" s="134"/>
+      <c r="J74" s="122"/>
+      <c r="L74" s="104"/>
+      <c r="M74" s="131"/>
+      <c r="N74" s="131"/>
+      <c r="O74" s="104"/>
+      <c r="Q74" s="137"/>
+      <c r="R74" s="137"/>
+      <c r="S74" s="137"/>
     </row>
     <row r="75" spans="1:20" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="D75" s="64"/>
-      <c r="E75" s="67"/>
-      <c r="G75" s="61"/>
-      <c r="H75" s="76"/>
-      <c r="I75" s="76"/>
-      <c r="J75" s="61"/>
-      <c r="L75" s="70"/>
-      <c r="M75" s="73"/>
-      <c r="N75" s="73"/>
-      <c r="O75" s="70"/>
-      <c r="Q75" s="79"/>
-      <c r="R75" s="79"/>
-      <c r="S75" s="79"/>
+      <c r="D75" s="126"/>
+      <c r="E75" s="129"/>
+      <c r="G75" s="123"/>
+      <c r="H75" s="135"/>
+      <c r="I75" s="135"/>
+      <c r="J75" s="123"/>
+      <c r="L75" s="105"/>
+      <c r="M75" s="132"/>
+      <c r="N75" s="132"/>
+      <c r="O75" s="105"/>
+      <c r="Q75" s="138"/>
+      <c r="R75" s="138"/>
+      <c r="S75" s="138"/>
     </row>
   </sheetData>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B6:T60">
     <sortCondition ref="B6"/>
   </sortState>
   <mergeCells count="25">
-    <mergeCell ref="G2:K2"/>
-    <mergeCell ref="D2:F2"/>
-    <mergeCell ref="Q3:T4"/>
-    <mergeCell ref="O66:O75"/>
-    <mergeCell ref="A2:A5"/>
-    <mergeCell ref="G3:K4"/>
-    <mergeCell ref="D3:F4"/>
-    <mergeCell ref="B2:B5"/>
-    <mergeCell ref="C2:C5"/>
     <mergeCell ref="B1:T1"/>
     <mergeCell ref="J66:J75"/>
     <mergeCell ref="D66:D75"/>
@@ -7764,6 +7757,15 @@
     <mergeCell ref="I66:I75"/>
     <mergeCell ref="Q2:T2"/>
     <mergeCell ref="L2:P2"/>
+    <mergeCell ref="G2:K2"/>
+    <mergeCell ref="D2:F2"/>
+    <mergeCell ref="Q3:T4"/>
+    <mergeCell ref="O66:O75"/>
+    <mergeCell ref="A2:A5"/>
+    <mergeCell ref="G3:K4"/>
+    <mergeCell ref="D3:F4"/>
+    <mergeCell ref="B2:B5"/>
+    <mergeCell ref="C2:C5"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
me siento orgulloso de mi y de mi esposa
</commit_message>
<xml_diff>
--- a/9_asistencia_evaluacion/pivu_caucasia.xlsx
+++ b/9_asistencia_evaluacion/pivu_caucasia.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\marco\Documentos\extension\camino-udea\9_asistencia_evaluacion\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{70D4DA88-E0DF-4EB6-93CF-45B1295C9DB5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{08F52304-9FD3-429F-B0D7-1759AD04E300}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1136,6 +1136,90 @@
     <xf numFmtId="0" fontId="22" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="14" fillId="11" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1163,15 +1247,6 @@
     <xf numFmtId="0" fontId="3" fillId="7" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="9" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1212,81 +1287,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="6" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="8" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="9" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="8" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="9" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="9" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="9" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="9" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="9" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="9" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -3002,14 +3002,14 @@
         <v>1038117202</v>
       </c>
       <c r="D7" s="13">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E7" s="13"/>
       <c r="F7" s="13"/>
       <c r="G7" s="13"/>
       <c r="H7" s="32">
         <f t="shared" ref="H7:H40" si="0">+SUM(D7:G7)/4</f>
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="I7" s="33"/>
       <c r="J7" s="33"/>
@@ -3057,14 +3057,14 @@
         <v>1041633525</v>
       </c>
       <c r="D8" s="13">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E8" s="13"/>
       <c r="F8" s="13"/>
       <c r="G8" s="13"/>
       <c r="H8" s="32">
         <f t="shared" si="0"/>
-        <v>1.25</v>
+        <v>1.5</v>
       </c>
       <c r="I8" s="33"/>
       <c r="J8" s="33"/>
@@ -3222,14 +3222,14 @@
         <v>1038110143</v>
       </c>
       <c r="D11" s="13">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E11" s="13"/>
       <c r="F11" s="13"/>
       <c r="G11" s="13"/>
       <c r="H11" s="32">
         <f t="shared" si="0"/>
-        <v>1</v>
+        <v>1.25</v>
       </c>
       <c r="I11" s="33"/>
       <c r="J11" s="33"/>
@@ -3332,14 +3332,14 @@
         <v>1038116790</v>
       </c>
       <c r="D13" s="13">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E13" s="13"/>
       <c r="F13" s="13"/>
       <c r="G13" s="13"/>
       <c r="H13" s="32">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>0.25</v>
       </c>
       <c r="I13" s="33"/>
       <c r="J13" s="33"/>
@@ -3387,14 +3387,14 @@
         <v>1038111245</v>
       </c>
       <c r="D14" s="13">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E14" s="13"/>
       <c r="F14" s="13"/>
       <c r="G14" s="13"/>
       <c r="H14" s="32">
         <f t="shared" si="0"/>
-        <v>2</v>
+        <v>2.25</v>
       </c>
       <c r="I14" s="33"/>
       <c r="J14" s="33"/>
@@ -3442,14 +3442,14 @@
         <v>1038134078</v>
       </c>
       <c r="D15" s="13">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E15" s="13"/>
       <c r="F15" s="13"/>
       <c r="G15" s="13"/>
       <c r="H15" s="32">
         <f t="shared" si="0"/>
-        <v>0.75</v>
+        <v>1</v>
       </c>
       <c r="I15" s="33"/>
       <c r="J15" s="33"/>
@@ -3717,14 +3717,14 @@
         <v>1038105559</v>
       </c>
       <c r="D20" s="13">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E20" s="13"/>
       <c r="F20" s="13"/>
       <c r="G20" s="13"/>
       <c r="H20" s="32">
         <f t="shared" si="0"/>
-        <v>1.25</v>
+        <v>1.5</v>
       </c>
       <c r="I20" s="33"/>
       <c r="J20" s="33"/>
@@ -3882,14 +3882,14 @@
         <v>1038113598</v>
       </c>
       <c r="D23" s="13">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E23" s="13"/>
       <c r="F23" s="13"/>
       <c r="G23" s="13"/>
       <c r="H23" s="32">
         <f t="shared" si="0"/>
-        <v>0.5</v>
+        <v>0.75</v>
       </c>
       <c r="I23" s="33"/>
       <c r="J23" s="33"/>
@@ -3937,14 +3937,14 @@
         <v>1038648337</v>
       </c>
       <c r="D24" s="13">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E24" s="13"/>
       <c r="F24" s="13"/>
       <c r="G24" s="13"/>
       <c r="H24" s="32">
         <f t="shared" si="0"/>
-        <v>0.25</v>
+        <v>0.5</v>
       </c>
       <c r="I24" s="33"/>
       <c r="J24" s="33"/>
@@ -4046,7 +4046,9 @@
         <f>+Inscritos!D24</f>
         <v>1066518419</v>
       </c>
-      <c r="D26" s="13"/>
+      <c r="D26" s="13">
+        <v>0</v>
+      </c>
       <c r="E26" s="13"/>
       <c r="F26" s="13"/>
       <c r="G26" s="13"/>
@@ -4210,14 +4212,14 @@
         <v>1038109706</v>
       </c>
       <c r="D29" s="13">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E29" s="13"/>
       <c r="F29" s="13"/>
       <c r="G29" s="13"/>
       <c r="H29" s="32">
         <f t="shared" si="0"/>
-        <v>1.25</v>
+        <v>1.5</v>
       </c>
       <c r="I29" s="33"/>
       <c r="J29" s="33"/>
@@ -4375,14 +4377,14 @@
         <v>1038104210</v>
       </c>
       <c r="D32" s="13">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E32" s="13"/>
       <c r="F32" s="13"/>
       <c r="G32" s="13"/>
       <c r="H32" s="32">
         <f t="shared" si="0"/>
-        <v>2.25</v>
+        <v>2.5</v>
       </c>
       <c r="I32" s="33"/>
       <c r="J32" s="33"/>
@@ -4540,14 +4542,14 @@
         <v>1038115337</v>
       </c>
       <c r="D35" s="13">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E35" s="13"/>
       <c r="F35" s="13"/>
       <c r="G35" s="13"/>
       <c r="H35" s="32">
         <f t="shared" si="0"/>
-        <v>1.25</v>
+        <v>1.5</v>
       </c>
       <c r="I35" s="33"/>
       <c r="J35" s="33"/>
@@ -4595,14 +4597,14 @@
         <v>1116074065</v>
       </c>
       <c r="D36" s="13">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E36" s="13"/>
       <c r="F36" s="13"/>
       <c r="G36" s="13"/>
       <c r="H36" s="32">
         <f t="shared" si="0"/>
-        <v>0.75</v>
+        <v>0.25</v>
       </c>
       <c r="I36" s="33"/>
       <c r="J36" s="33"/>
@@ -4760,14 +4762,14 @@
         <v>1038113397</v>
       </c>
       <c r="D39" s="13">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E39" s="13"/>
       <c r="F39" s="13"/>
       <c r="G39" s="13"/>
       <c r="H39" s="32">
         <f t="shared" si="0"/>
-        <v>0.75</v>
+        <v>1</v>
       </c>
       <c r="I39" s="33"/>
       <c r="J39" s="33"/>
@@ -4810,11 +4812,11 @@
         <v>105</v>
       </c>
       <c r="D40" s="57">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H40" s="2">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>0.25</v>
       </c>
     </row>
   </sheetData>
@@ -4869,30 +4871,30 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:20" ht="72.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B1" s="120" t="s">
+      <c r="B1" s="94" t="s">
         <v>18</v>
       </c>
-      <c r="C1" s="120"/>
-      <c r="D1" s="120"/>
-      <c r="E1" s="120"/>
-      <c r="F1" s="120"/>
-      <c r="G1" s="120"/>
-      <c r="H1" s="120"/>
-      <c r="I1" s="120"/>
-      <c r="J1" s="120"/>
-      <c r="K1" s="120"/>
-      <c r="L1" s="120"/>
-      <c r="M1" s="120"/>
-      <c r="N1" s="120"/>
-      <c r="O1" s="120"/>
-      <c r="P1" s="120"/>
-      <c r="Q1" s="120"/>
-      <c r="R1" s="120"/>
-      <c r="S1" s="120"/>
-      <c r="T1" s="120"/>
+      <c r="C1" s="94"/>
+      <c r="D1" s="94"/>
+      <c r="E1" s="94"/>
+      <c r="F1" s="94"/>
+      <c r="G1" s="94"/>
+      <c r="H1" s="94"/>
+      <c r="I1" s="94"/>
+      <c r="J1" s="94"/>
+      <c r="K1" s="94"/>
+      <c r="L1" s="94"/>
+      <c r="M1" s="94"/>
+      <c r="N1" s="94"/>
+      <c r="O1" s="94"/>
+      <c r="P1" s="94"/>
+      <c r="Q1" s="94"/>
+      <c r="R1" s="94"/>
+      <c r="S1" s="94"/>
+      <c r="T1" s="94"/>
     </row>
     <row r="2" spans="1:20" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A2" s="106" t="s">
+      <c r="A2" s="131" t="s">
         <v>13</v>
       </c>
       <c r="B2" s="90" t="s">
@@ -4901,89 +4903,89 @@
       <c r="C2" s="66" t="s">
         <v>3</v>
       </c>
-      <c r="D2" s="94" t="str">
+      <c r="D2" s="122" t="str">
         <f>Asistencia!D2</f>
         <v>NOMBRE DOCENTE</v>
       </c>
-      <c r="E2" s="95"/>
-      <c r="F2" s="96"/>
-      <c r="G2" s="94" t="str">
+      <c r="E2" s="123"/>
+      <c r="F2" s="124"/>
+      <c r="G2" s="122" t="str">
         <f>Asistencia!I2</f>
         <v>NOMBRE DOCENTE</v>
       </c>
-      <c r="H2" s="95"/>
-      <c r="I2" s="95"/>
-      <c r="J2" s="95"/>
-      <c r="K2" s="96"/>
-      <c r="L2" s="94" t="s">
+      <c r="H2" s="123"/>
+      <c r="I2" s="123"/>
+      <c r="J2" s="123"/>
+      <c r="K2" s="124"/>
+      <c r="L2" s="122" t="s">
         <v>19</v>
       </c>
-      <c r="M2" s="95"/>
-      <c r="N2" s="95"/>
-      <c r="O2" s="95"/>
-      <c r="P2" s="96"/>
-      <c r="Q2" s="94" t="str">
+      <c r="M2" s="123"/>
+      <c r="N2" s="123"/>
+      <c r="O2" s="123"/>
+      <c r="P2" s="124"/>
+      <c r="Q2" s="122" t="str">
         <f>Asistencia!AA2</f>
         <v>NOMBRE DOCENTE</v>
       </c>
-      <c r="R2" s="95"/>
-      <c r="S2" s="95"/>
-      <c r="T2" s="96"/>
+      <c r="R2" s="123"/>
+      <c r="S2" s="123"/>
+      <c r="T2" s="124"/>
     </row>
     <row r="3" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="107"/>
+      <c r="A3" s="132"/>
       <c r="B3" s="91"/>
       <c r="C3" s="67"/>
-      <c r="D3" s="114" t="s">
+      <c r="D3" s="139" t="s">
         <v>7</v>
       </c>
-      <c r="E3" s="115"/>
-      <c r="F3" s="116"/>
-      <c r="G3" s="108" t="s">
+      <c r="E3" s="140"/>
+      <c r="F3" s="141"/>
+      <c r="G3" s="133" t="s">
         <v>2</v>
       </c>
-      <c r="H3" s="109"/>
-      <c r="I3" s="109"/>
-      <c r="J3" s="109"/>
-      <c r="K3" s="110"/>
-      <c r="L3" s="139" t="s">
+      <c r="H3" s="134"/>
+      <c r="I3" s="134"/>
+      <c r="J3" s="134"/>
+      <c r="K3" s="135"/>
+      <c r="L3" s="116" t="s">
         <v>1</v>
       </c>
-      <c r="M3" s="140"/>
-      <c r="N3" s="140"/>
-      <c r="O3" s="140"/>
-      <c r="P3" s="141"/>
-      <c r="Q3" s="97" t="s">
-        <v>0</v>
-      </c>
-      <c r="R3" s="98"/>
-      <c r="S3" s="98"/>
-      <c r="T3" s="99"/>
+      <c r="M3" s="117"/>
+      <c r="N3" s="117"/>
+      <c r="O3" s="117"/>
+      <c r="P3" s="118"/>
+      <c r="Q3" s="125" t="s">
+        <v>0</v>
+      </c>
+      <c r="R3" s="126"/>
+      <c r="S3" s="126"/>
+      <c r="T3" s="127"/>
     </row>
     <row r="4" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="107"/>
+      <c r="A4" s="132"/>
       <c r="B4" s="91"/>
       <c r="C4" s="67"/>
-      <c r="D4" s="117"/>
-      <c r="E4" s="118"/>
-      <c r="F4" s="119"/>
-      <c r="G4" s="111"/>
-      <c r="H4" s="112"/>
-      <c r="I4" s="112"/>
-      <c r="J4" s="112"/>
-      <c r="K4" s="113"/>
-      <c r="L4" s="142"/>
-      <c r="M4" s="143"/>
-      <c r="N4" s="143"/>
-      <c r="O4" s="143"/>
-      <c r="P4" s="144"/>
-      <c r="Q4" s="100"/>
-      <c r="R4" s="101"/>
-      <c r="S4" s="101"/>
-      <c r="T4" s="102"/>
+      <c r="D4" s="142"/>
+      <c r="E4" s="143"/>
+      <c r="F4" s="144"/>
+      <c r="G4" s="136"/>
+      <c r="H4" s="137"/>
+      <c r="I4" s="137"/>
+      <c r="J4" s="137"/>
+      <c r="K4" s="138"/>
+      <c r="L4" s="119"/>
+      <c r="M4" s="120"/>
+      <c r="N4" s="120"/>
+      <c r="O4" s="120"/>
+      <c r="P4" s="121"/>
+      <c r="Q4" s="128"/>
+      <c r="R4" s="129"/>
+      <c r="S4" s="129"/>
+      <c r="T4" s="130"/>
     </row>
     <row r="5" spans="1:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="107"/>
+      <c r="A5" s="132"/>
       <c r="B5" s="91"/>
       <c r="C5" s="67"/>
       <c r="D5" s="17">
@@ -7561,186 +7563,195 @@
       </c>
     </row>
     <row r="66" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="D66" s="124" t="s">
+      <c r="D66" s="98" t="s">
         <v>24</v>
       </c>
-      <c r="E66" s="127" t="s">
+      <c r="E66" s="101" t="s">
         <v>12</v>
       </c>
-      <c r="G66" s="121" t="s">
+      <c r="G66" s="95" t="s">
         <v>8</v>
       </c>
-      <c r="H66" s="133" t="s">
+      <c r="H66" s="110" t="s">
         <v>9</v>
       </c>
-      <c r="I66" s="133" t="s">
+      <c r="I66" s="110" t="s">
         <v>10</v>
       </c>
-      <c r="J66" s="121" t="s">
+      <c r="J66" s="95" t="s">
         <v>11</v>
       </c>
-      <c r="L66" s="103" t="s">
+      <c r="L66" s="104" t="s">
         <v>8</v>
       </c>
-      <c r="M66" s="130" t="s">
+      <c r="M66" s="107" t="s">
         <v>9</v>
       </c>
-      <c r="N66" s="130" t="s">
+      <c r="N66" s="107" t="s">
         <v>10</v>
       </c>
-      <c r="O66" s="103" t="s">
+      <c r="O66" s="104" t="s">
         <v>11</v>
       </c>
-      <c r="Q66" s="136" t="s">
+      <c r="Q66" s="113" t="s">
         <v>24</v>
       </c>
-      <c r="R66" s="136" t="s">
+      <c r="R66" s="113" t="s">
         <v>4</v>
       </c>
-      <c r="S66" s="136" t="s">
+      <c r="S66" s="113" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="67" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="D67" s="125"/>
-      <c r="E67" s="128"/>
-      <c r="G67" s="122"/>
-      <c r="H67" s="134"/>
-      <c r="I67" s="134"/>
-      <c r="J67" s="122"/>
-      <c r="L67" s="104"/>
-      <c r="M67" s="131"/>
-      <c r="N67" s="131"/>
-      <c r="O67" s="104"/>
-      <c r="Q67" s="137"/>
-      <c r="R67" s="137"/>
-      <c r="S67" s="137"/>
+      <c r="D67" s="99"/>
+      <c r="E67" s="102"/>
+      <c r="G67" s="96"/>
+      <c r="H67" s="111"/>
+      <c r="I67" s="111"/>
+      <c r="J67" s="96"/>
+      <c r="L67" s="105"/>
+      <c r="M67" s="108"/>
+      <c r="N67" s="108"/>
+      <c r="O67" s="105"/>
+      <c r="Q67" s="114"/>
+      <c r="R67" s="114"/>
+      <c r="S67" s="114"/>
     </row>
     <row r="68" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="D68" s="125"/>
-      <c r="E68" s="128"/>
-      <c r="G68" s="122"/>
-      <c r="H68" s="134"/>
-      <c r="I68" s="134"/>
-      <c r="J68" s="122"/>
-      <c r="L68" s="104"/>
-      <c r="M68" s="131"/>
-      <c r="N68" s="131"/>
-      <c r="O68" s="104"/>
-      <c r="Q68" s="137"/>
-      <c r="R68" s="137"/>
-      <c r="S68" s="137"/>
+      <c r="D68" s="99"/>
+      <c r="E68" s="102"/>
+      <c r="G68" s="96"/>
+      <c r="H68" s="111"/>
+      <c r="I68" s="111"/>
+      <c r="J68" s="96"/>
+      <c r="L68" s="105"/>
+      <c r="M68" s="108"/>
+      <c r="N68" s="108"/>
+      <c r="O68" s="105"/>
+      <c r="Q68" s="114"/>
+      <c r="R68" s="114"/>
+      <c r="S68" s="114"/>
     </row>
     <row r="69" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="D69" s="125"/>
-      <c r="E69" s="128"/>
-      <c r="G69" s="122"/>
-      <c r="H69" s="134"/>
-      <c r="I69" s="134"/>
-      <c r="J69" s="122"/>
-      <c r="L69" s="104"/>
-      <c r="M69" s="131"/>
-      <c r="N69" s="131"/>
-      <c r="O69" s="104"/>
-      <c r="Q69" s="137"/>
-      <c r="R69" s="137"/>
-      <c r="S69" s="137"/>
+      <c r="D69" s="99"/>
+      <c r="E69" s="102"/>
+      <c r="G69" s="96"/>
+      <c r="H69" s="111"/>
+      <c r="I69" s="111"/>
+      <c r="J69" s="96"/>
+      <c r="L69" s="105"/>
+      <c r="M69" s="108"/>
+      <c r="N69" s="108"/>
+      <c r="O69" s="105"/>
+      <c r="Q69" s="114"/>
+      <c r="R69" s="114"/>
+      <c r="S69" s="114"/>
     </row>
     <row r="70" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="D70" s="125"/>
-      <c r="E70" s="128"/>
-      <c r="G70" s="122"/>
-      <c r="H70" s="134"/>
-      <c r="I70" s="134"/>
-      <c r="J70" s="122"/>
-      <c r="L70" s="104"/>
-      <c r="M70" s="131"/>
-      <c r="N70" s="131"/>
-      <c r="O70" s="104"/>
-      <c r="Q70" s="137"/>
-      <c r="R70" s="137"/>
-      <c r="S70" s="137"/>
+      <c r="D70" s="99"/>
+      <c r="E70" s="102"/>
+      <c r="G70" s="96"/>
+      <c r="H70" s="111"/>
+      <c r="I70" s="111"/>
+      <c r="J70" s="96"/>
+      <c r="L70" s="105"/>
+      <c r="M70" s="108"/>
+      <c r="N70" s="108"/>
+      <c r="O70" s="105"/>
+      <c r="Q70" s="114"/>
+      <c r="R70" s="114"/>
+      <c r="S70" s="114"/>
     </row>
     <row r="71" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="D71" s="125"/>
-      <c r="E71" s="128"/>
-      <c r="G71" s="122"/>
-      <c r="H71" s="134"/>
-      <c r="I71" s="134"/>
-      <c r="J71" s="122"/>
-      <c r="L71" s="104"/>
-      <c r="M71" s="131"/>
-      <c r="N71" s="131"/>
-      <c r="O71" s="104"/>
-      <c r="Q71" s="137"/>
-      <c r="R71" s="137"/>
-      <c r="S71" s="137"/>
+      <c r="D71" s="99"/>
+      <c r="E71" s="102"/>
+      <c r="G71" s="96"/>
+      <c r="H71" s="111"/>
+      <c r="I71" s="111"/>
+      <c r="J71" s="96"/>
+      <c r="L71" s="105"/>
+      <c r="M71" s="108"/>
+      <c r="N71" s="108"/>
+      <c r="O71" s="105"/>
+      <c r="Q71" s="114"/>
+      <c r="R71" s="114"/>
+      <c r="S71" s="114"/>
     </row>
     <row r="72" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="D72" s="125"/>
-      <c r="E72" s="128"/>
-      <c r="G72" s="122"/>
-      <c r="H72" s="134"/>
-      <c r="I72" s="134"/>
-      <c r="J72" s="122"/>
-      <c r="L72" s="104"/>
-      <c r="M72" s="131"/>
-      <c r="N72" s="131"/>
-      <c r="O72" s="104"/>
-      <c r="Q72" s="137"/>
-      <c r="R72" s="137"/>
-      <c r="S72" s="137"/>
+      <c r="D72" s="99"/>
+      <c r="E72" s="102"/>
+      <c r="G72" s="96"/>
+      <c r="H72" s="111"/>
+      <c r="I72" s="111"/>
+      <c r="J72" s="96"/>
+      <c r="L72" s="105"/>
+      <c r="M72" s="108"/>
+      <c r="N72" s="108"/>
+      <c r="O72" s="105"/>
+      <c r="Q72" s="114"/>
+      <c r="R72" s="114"/>
+      <c r="S72" s="114"/>
     </row>
     <row r="73" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="D73" s="125"/>
-      <c r="E73" s="128"/>
-      <c r="G73" s="122"/>
-      <c r="H73" s="134"/>
-      <c r="I73" s="134"/>
-      <c r="J73" s="122"/>
-      <c r="L73" s="104"/>
-      <c r="M73" s="131"/>
-      <c r="N73" s="131"/>
-      <c r="O73" s="104"/>
-      <c r="Q73" s="137"/>
-      <c r="R73" s="137"/>
-      <c r="S73" s="137"/>
+      <c r="D73" s="99"/>
+      <c r="E73" s="102"/>
+      <c r="G73" s="96"/>
+      <c r="H73" s="111"/>
+      <c r="I73" s="111"/>
+      <c r="J73" s="96"/>
+      <c r="L73" s="105"/>
+      <c r="M73" s="108"/>
+      <c r="N73" s="108"/>
+      <c r="O73" s="105"/>
+      <c r="Q73" s="114"/>
+      <c r="R73" s="114"/>
+      <c r="S73" s="114"/>
     </row>
     <row r="74" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="D74" s="125"/>
-      <c r="E74" s="128"/>
-      <c r="G74" s="122"/>
-      <c r="H74" s="134"/>
-      <c r="I74" s="134"/>
-      <c r="J74" s="122"/>
-      <c r="L74" s="104"/>
-      <c r="M74" s="131"/>
-      <c r="N74" s="131"/>
-      <c r="O74" s="104"/>
-      <c r="Q74" s="137"/>
-      <c r="R74" s="137"/>
-      <c r="S74" s="137"/>
+      <c r="D74" s="99"/>
+      <c r="E74" s="102"/>
+      <c r="G74" s="96"/>
+      <c r="H74" s="111"/>
+      <c r="I74" s="111"/>
+      <c r="J74" s="96"/>
+      <c r="L74" s="105"/>
+      <c r="M74" s="108"/>
+      <c r="N74" s="108"/>
+      <c r="O74" s="105"/>
+      <c r="Q74" s="114"/>
+      <c r="R74" s="114"/>
+      <c r="S74" s="114"/>
     </row>
     <row r="75" spans="1:20" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="D75" s="126"/>
-      <c r="E75" s="129"/>
-      <c r="G75" s="123"/>
-      <c r="H75" s="135"/>
-      <c r="I75" s="135"/>
-      <c r="J75" s="123"/>
-      <c r="L75" s="105"/>
-      <c r="M75" s="132"/>
-      <c r="N75" s="132"/>
-      <c r="O75" s="105"/>
-      <c r="Q75" s="138"/>
-      <c r="R75" s="138"/>
-      <c r="S75" s="138"/>
+      <c r="D75" s="100"/>
+      <c r="E75" s="103"/>
+      <c r="G75" s="97"/>
+      <c r="H75" s="112"/>
+      <c r="I75" s="112"/>
+      <c r="J75" s="97"/>
+      <c r="L75" s="106"/>
+      <c r="M75" s="109"/>
+      <c r="N75" s="109"/>
+      <c r="O75" s="106"/>
+      <c r="Q75" s="115"/>
+      <c r="R75" s="115"/>
+      <c r="S75" s="115"/>
     </row>
   </sheetData>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B6:T60">
     <sortCondition ref="B6"/>
   </sortState>
   <mergeCells count="25">
+    <mergeCell ref="G2:K2"/>
+    <mergeCell ref="D2:F2"/>
+    <mergeCell ref="Q3:T4"/>
+    <mergeCell ref="O66:O75"/>
+    <mergeCell ref="A2:A5"/>
+    <mergeCell ref="G3:K4"/>
+    <mergeCell ref="D3:F4"/>
+    <mergeCell ref="B2:B5"/>
+    <mergeCell ref="C2:C5"/>
     <mergeCell ref="B1:T1"/>
     <mergeCell ref="J66:J75"/>
     <mergeCell ref="D66:D75"/>
@@ -7757,15 +7768,6 @@
     <mergeCell ref="I66:I75"/>
     <mergeCell ref="Q2:T2"/>
     <mergeCell ref="L2:P2"/>
-    <mergeCell ref="G2:K2"/>
-    <mergeCell ref="D2:F2"/>
-    <mergeCell ref="Q3:T4"/>
-    <mergeCell ref="O66:O75"/>
-    <mergeCell ref="A2:A5"/>
-    <mergeCell ref="G3:K4"/>
-    <mergeCell ref="D3:F4"/>
-    <mergeCell ref="B2:B5"/>
-    <mergeCell ref="C2:C5"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>